<commit_message>
Update README and command reference Excel with stock list command
Add `stock list` to README examples, command table, and reference
section. Update Excel (220 commands, stock count 58).

https://claude.ai/code/session_01Bw7ybw8i1cDGBDXFVaPJ8Z
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$220</definedName>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H220"/>
+  <dimension ref="A1:H221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8578,90 +8578,87 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="12" t="inlineStr">
+      <c r="A191" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B191" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C191" s="12" t="inlineStr">
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>list</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>kiwoom stock list</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>KRX 전체 상장종목 리스트 (pykrx)</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>--market [all, kospi, kosdaq, konex] 기본:all (시장구분)
+--search (종목명/코드 검색 키워드)
+--refresh (캐시 무시하고 새로 조회)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B192" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C192" s="12" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="D191" s="12" t="inlineStr">
+      <c r="D192" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock short</t>
         </is>
       </c>
-      <c r="E191" s="12" t="inlineStr">
+      <c r="E192" s="12" t="inlineStr">
         <is>
           <t>공매도 추이 조회</t>
         </is>
       </c>
-      <c r="F191" s="13" t="inlineStr">
+      <c r="F192" s="13" t="inlineStr">
         <is>
           <t>ka10014</t>
         </is>
       </c>
-      <c r="G191" s="12" t="inlineStr">
+      <c r="G192" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H191" s="12" t="inlineStr">
+      <c r="H192" s="12" t="inlineStr">
         <is>
           <t>--from (시작일자 (YYYYMMDD, 기본=30일전))
 --to (종료일자 (YYYYMMDD, 기본=오늘))</t>
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B192" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C192" s="12" t="inlineStr">
-        <is>
-          <t>tick-strength</t>
-        </is>
-      </c>
-      <c r="D192" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock tick-strength</t>
-        </is>
-      </c>
-      <c r="E192" s="12" t="inlineStr">
-        <is>
-          <t>체결강도추이 시간별</t>
-        </is>
-      </c>
-      <c r="F192" s="13" t="inlineStr">
-        <is>
-          <t>ka10046</t>
-        </is>
-      </c>
-      <c r="G192" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H192" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
     <row r="193">
       <c r="A193" s="12" t="inlineStr">
         <is>
@@ -8675,22 +8672,22 @@
       </c>
       <c r="C193" s="12" t="inlineStr">
         <is>
-          <t>timeprice</t>
+          <t>tick-strength</t>
         </is>
       </c>
       <c r="D193" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock timeprice</t>
+          <t>kiwoom stock tick-strength</t>
         </is>
       </c>
       <c r="E193" s="12" t="inlineStr">
         <is>
-          <t>시분 시세 조회</t>
+          <t>체결강도추이 시간별</t>
         </is>
       </c>
       <c r="F193" s="13" t="inlineStr">
         <is>
-          <t>ka10006</t>
+          <t>ka10046</t>
         </is>
       </c>
       <c r="G193" s="12" t="inlineStr">
@@ -8717,30 +8714,72 @@
       </c>
       <c r="C194" s="12" t="inlineStr">
         <is>
+          <t>timeprice</t>
+        </is>
+      </c>
+      <c r="D194" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock timeprice</t>
+        </is>
+      </c>
+      <c r="E194" s="12" t="inlineStr">
+        <is>
+          <t>시분 시세 조회</t>
+        </is>
+      </c>
+      <c r="F194" s="13" t="inlineStr">
+        <is>
+          <t>ka10006</t>
+        </is>
+      </c>
+      <c r="G194" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H194" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B195" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C195" s="12" t="inlineStr">
+        <is>
           <t>today-exec</t>
         </is>
       </c>
-      <c r="D194" s="12" t="inlineStr">
+      <c r="D195" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock today-exec</t>
         </is>
       </c>
-      <c r="E194" s="12" t="inlineStr">
+      <c r="E195" s="12" t="inlineStr">
         <is>
           <t>당일/전일 체결 조회</t>
         </is>
       </c>
-      <c r="F194" s="13" t="inlineStr">
+      <c r="F195" s="13" t="inlineStr">
         <is>
           <t>ka10084</t>
         </is>
       </c>
-      <c r="G194" s="12" t="inlineStr">
+      <c r="G195" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H194" s="12" t="inlineStr">
+      <c r="H195" s="12" t="inlineStr">
         <is>
           <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))
 --mode [0, 1] (틱/분 (0=틱, 1=분))
@@ -8748,48 +8787,6 @@
         </is>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B195" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C195" s="12" t="inlineStr">
-        <is>
-          <t>today-volume</t>
-        </is>
-      </c>
-      <c r="D195" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock today-volume</t>
-        </is>
-      </c>
-      <c r="E195" s="12" t="inlineStr">
-        <is>
-          <t>당일/전일 체결량 조회</t>
-        </is>
-      </c>
-      <c r="F195" s="13" t="inlineStr">
-        <is>
-          <t>ka10055</t>
-        </is>
-      </c>
-      <c r="G195" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H195" s="12" t="inlineStr">
-        <is>
-          <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))</t>
-        </is>
-      </c>
-    </row>
     <row r="196">
       <c r="A196" s="12" t="inlineStr">
         <is>
@@ -8803,22 +8800,22 @@
       </c>
       <c r="C196" s="12" t="inlineStr">
         <is>
-          <t>trader</t>
+          <t>today-volume</t>
         </is>
       </c>
       <c r="D196" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock trader</t>
+          <t>kiwoom stock today-volume</t>
         </is>
       </c>
       <c r="E196" s="12" t="inlineStr">
         <is>
-          <t>거래원 조회</t>
+          <t>당일/전일 체결량 조회</t>
         </is>
       </c>
       <c r="F196" s="13" t="inlineStr">
         <is>
-          <t>ka10002</t>
+          <t>ka10055</t>
         </is>
       </c>
       <c r="G196" s="12" t="inlineStr">
@@ -8828,7 +8825,7 @@
       </c>
       <c r="H196" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))</t>
         </is>
       </c>
     </row>
@@ -8845,70 +8842,74 @@
       </c>
       <c r="C197" s="12" t="inlineStr">
         <is>
+          <t>trader</t>
+        </is>
+      </c>
+      <c r="D197" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock trader</t>
+        </is>
+      </c>
+      <c r="E197" s="12" t="inlineStr">
+        <is>
+          <t>거래원 조회</t>
+        </is>
+      </c>
+      <c r="F197" s="13" t="inlineStr">
+        <is>
+          <t>ka10002</t>
+        </is>
+      </c>
+      <c r="G197" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H197" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B198" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C198" s="12" t="inlineStr">
+        <is>
           <t>watchlist</t>
         </is>
       </c>
-      <c r="D197" s="12" t="inlineStr">
+      <c r="D198" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock watchlist</t>
         </is>
       </c>
-      <c r="E197" s="12" t="inlineStr">
+      <c r="E198" s="12" t="inlineStr">
         <is>
           <t>관심종목정보 조회 (코드를 |로 구분, 예: 005930|000660)</t>
         </is>
       </c>
-      <c r="F197" s="13" t="inlineStr">
+      <c r="F198" s="13" t="inlineStr">
         <is>
           <t>ka10095</t>
         </is>
       </c>
-      <c r="G197" s="12" t="inlineStr">
+      <c r="G198" s="12" t="inlineStr">
         <is>
           <t>CODES (필수)</t>
         </is>
       </c>
-      <c r="H197" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="14" t="inlineStr">
-        <is>
-          <t>stream</t>
-        </is>
-      </c>
-      <c r="B198" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C198" s="14" t="inlineStr">
-        <is>
-          <t>after-hours</t>
-        </is>
-      </c>
-      <c r="D198" s="14" t="inlineStr">
-        <is>
-          <t>kiwoom stream after-hours</t>
-        </is>
-      </c>
-      <c r="E198" s="14" t="inlineStr">
-        <is>
-          <t>주식시간외호가 실시간 (0E)</t>
-        </is>
-      </c>
-      <c r="F198" s="15" t="inlineStr"/>
-      <c r="G198" s="14" t="inlineStr">
-        <is>
-          <t>CODES (복수) (필수)</t>
-        </is>
-      </c>
-      <c r="H198" s="14" t="inlineStr">
-        <is>
-          <t>--raw (JSON 원본 출력)</t>
+      <c r="H198" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -8925,23 +8926,23 @@
       </c>
       <c r="C199" s="14" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>after-hours</t>
         </is>
       </c>
       <c r="D199" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream balance</t>
+          <t>kiwoom stream after-hours</t>
         </is>
       </c>
       <c r="E199" s="14" t="inlineStr">
         <is>
-          <t>잔고 실시간 (04)</t>
+          <t>주식시간외호가 실시간 (0E)</t>
         </is>
       </c>
       <c r="F199" s="15" t="inlineStr"/>
       <c r="G199" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H199" s="14" t="inlineStr">
@@ -8963,23 +8964,23 @@
       </c>
       <c r="C200" s="14" t="inlineStr">
         <is>
-          <t>best-bid</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="D200" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream best-bid</t>
+          <t>kiwoom stream balance</t>
         </is>
       </c>
       <c r="E200" s="14" t="inlineStr">
         <is>
-          <t>주식우선호가 실시간 (0C)</t>
+          <t>잔고 실시간 (04)</t>
         </is>
       </c>
       <c r="F200" s="15" t="inlineStr"/>
       <c r="G200" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H200" s="14" t="inlineStr">
@@ -9001,64 +9002,64 @@
       </c>
       <c r="C201" s="14" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>best-bid</t>
         </is>
       </c>
       <c r="D201" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream custom</t>
+          <t>kiwoom stream best-bid</t>
         </is>
       </c>
       <c r="E201" s="14" t="inlineStr">
         <is>
-          <t>커스텀 실시간 타입으로 스트리밍</t>
+          <t>주식우선호가 실시간 (0C)</t>
         </is>
       </c>
       <c r="F201" s="15" t="inlineStr"/>
       <c r="G201" s="14" t="inlineStr">
         <is>
+          <t>CODES (복수) (필수)</t>
+        </is>
+      </c>
+      <c r="H201" s="14" t="inlineStr">
+        <is>
+          <t>--raw (JSON 원본 출력)</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="14" t="inlineStr">
+        <is>
+          <t>stream</t>
+        </is>
+      </c>
+      <c r="B202" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C202" s="14" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="D202" s="14" t="inlineStr">
+        <is>
+          <t>kiwoom stream custom</t>
+        </is>
+      </c>
+      <c r="E202" s="14" t="inlineStr">
+        <is>
+          <t>커스텀 실시간 타입으로 스트리밍</t>
+        </is>
+      </c>
+      <c r="F202" s="15" t="inlineStr"/>
+      <c r="G202" s="14" t="inlineStr">
+        <is>
           <t>TYPE_CODES (필수)
 CODES (복수) (선택)</t>
         </is>
       </c>
-      <c r="H201" s="14" t="inlineStr">
-        <is>
-          <t>--raw (JSON 원본 출력)</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="14" t="inlineStr">
-        <is>
-          <t>stream</t>
-        </is>
-      </c>
-      <c r="B202" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C202" s="14" t="inlineStr">
-        <is>
-          <t>elw-indicator</t>
-        </is>
-      </c>
-      <c r="D202" s="14" t="inlineStr">
-        <is>
-          <t>kiwoom stream elw-indicator</t>
-        </is>
-      </c>
-      <c r="E202" s="14" t="inlineStr">
-        <is>
-          <t>ELW 지표 실시간 (0u)</t>
-        </is>
-      </c>
-      <c r="F202" s="15" t="inlineStr"/>
-      <c r="G202" s="14" t="inlineStr">
-        <is>
-          <t>CODES (복수) (필수)</t>
-        </is>
-      </c>
       <c r="H202" s="14" t="inlineStr">
         <is>
           <t>--raw (JSON 원본 출력)</t>
@@ -9078,17 +9079,17 @@
       </c>
       <c r="C203" s="14" t="inlineStr">
         <is>
-          <t>elw-theory</t>
+          <t>elw-indicator</t>
         </is>
       </c>
       <c r="D203" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream elw-theory</t>
+          <t>kiwoom stream elw-indicator</t>
         </is>
       </c>
       <c r="E203" s="14" t="inlineStr">
         <is>
-          <t>ELW 이론가 실시간 (0m)</t>
+          <t>ELW 지표 실시간 (0u)</t>
         </is>
       </c>
       <c r="F203" s="15" t="inlineStr"/>
@@ -9116,17 +9117,17 @@
       </c>
       <c r="C204" s="14" t="inlineStr">
         <is>
-          <t>etf-nav</t>
+          <t>elw-theory</t>
         </is>
       </c>
       <c r="D204" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream etf-nav</t>
+          <t>kiwoom stream elw-theory</t>
         </is>
       </c>
       <c r="E204" s="14" t="inlineStr">
         <is>
-          <t>ETF NAV 실시간 (0G)</t>
+          <t>ELW 이론가 실시간 (0m)</t>
         </is>
       </c>
       <c r="F204" s="15" t="inlineStr"/>
@@ -9154,17 +9155,17 @@
       </c>
       <c r="C205" s="14" t="inlineStr">
         <is>
-          <t>expected</t>
+          <t>etf-nav</t>
         </is>
       </c>
       <c r="D205" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream expected</t>
+          <t>kiwoom stream etf-nav</t>
         </is>
       </c>
       <c r="E205" s="14" t="inlineStr">
         <is>
-          <t>주식예상체결 실시간 (0H)</t>
+          <t>ETF NAV 실시간 (0G)</t>
         </is>
       </c>
       <c r="F205" s="15" t="inlineStr"/>
@@ -9192,17 +9193,17 @@
       </c>
       <c r="C206" s="14" t="inlineStr">
         <is>
-          <t>gold</t>
+          <t>expected</t>
         </is>
       </c>
       <c r="D206" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream gold</t>
+          <t>kiwoom stream expected</t>
         </is>
       </c>
       <c r="E206" s="14" t="inlineStr">
         <is>
-          <t>국제금환산가격 실시간 (0I)</t>
+          <t>주식예상체결 실시간 (0H)</t>
         </is>
       </c>
       <c r="F206" s="15" t="inlineStr"/>
@@ -9230,23 +9231,23 @@
       </c>
       <c r="C207" s="14" t="inlineStr">
         <is>
-          <t>market-time</t>
+          <t>gold</t>
         </is>
       </c>
       <c r="D207" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream market-time</t>
+          <t>kiwoom stream gold</t>
         </is>
       </c>
       <c r="E207" s="14" t="inlineStr">
         <is>
-          <t>장시작시간 실시간 (0s)</t>
+          <t>국제금환산가격 실시간 (0I)</t>
         </is>
       </c>
       <c r="F207" s="15" t="inlineStr"/>
       <c r="G207" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H207" s="14" t="inlineStr">
@@ -9268,23 +9269,23 @@
       </c>
       <c r="C208" s="14" t="inlineStr">
         <is>
-          <t>multi</t>
+          <t>market-time</t>
         </is>
       </c>
       <c r="D208" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream multi</t>
+          <t>kiwoom stream market-time</t>
         </is>
       </c>
       <c r="E208" s="14" t="inlineStr">
         <is>
-          <t>주식체결+호가잔량 동시 스트리밍 (0B+0D)</t>
+          <t>장시작시간 실시간 (0s)</t>
         </is>
       </c>
       <c r="F208" s="15" t="inlineStr"/>
       <c r="G208" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H208" s="14" t="inlineStr">
@@ -9306,23 +9307,23 @@
       </c>
       <c r="C209" s="14" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>multi</t>
         </is>
       </c>
       <c r="D209" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream order</t>
+          <t>kiwoom stream multi</t>
         </is>
       </c>
       <c r="E209" s="14" t="inlineStr">
         <is>
-          <t>주문체결 실시간 (00)</t>
+          <t>주식체결+호가잔량 동시 스트리밍 (0B+0D)</t>
         </is>
       </c>
       <c r="F209" s="15" t="inlineStr"/>
       <c r="G209" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H209" s="14" t="inlineStr">
@@ -9344,23 +9345,23 @@
       </c>
       <c r="C210" s="14" t="inlineStr">
         <is>
-          <t>orderbook</t>
+          <t>order</t>
         </is>
       </c>
       <c r="D210" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream orderbook</t>
+          <t>kiwoom stream order</t>
         </is>
       </c>
       <c r="E210" s="14" t="inlineStr">
         <is>
-          <t>주식호가잔량 실시간 (0D)</t>
+          <t>주문체결 실시간 (00)</t>
         </is>
       </c>
       <c r="F210" s="15" t="inlineStr"/>
       <c r="G210" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H210" s="14" t="inlineStr">
@@ -9382,17 +9383,17 @@
       </c>
       <c r="C211" s="14" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>orderbook</t>
         </is>
       </c>
       <c r="D211" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream price</t>
+          <t>kiwoom stream orderbook</t>
         </is>
       </c>
       <c r="E211" s="14" t="inlineStr">
         <is>
-          <t>주식기세 실시간 (0A)</t>
+          <t>주식호가잔량 실시간 (0D)</t>
         </is>
       </c>
       <c r="F211" s="15" t="inlineStr"/>
@@ -9420,17 +9421,17 @@
       </c>
       <c r="C212" s="14" t="inlineStr">
         <is>
-          <t>program</t>
+          <t>price</t>
         </is>
       </c>
       <c r="D212" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream program</t>
+          <t>kiwoom stream price</t>
         </is>
       </c>
       <c r="E212" s="14" t="inlineStr">
         <is>
-          <t>종목프로그램매매 실시간 (0w)</t>
+          <t>주식기세 실시간 (0A)</t>
         </is>
       </c>
       <c r="F212" s="15" t="inlineStr"/>
@@ -9458,17 +9459,17 @@
       </c>
       <c r="C213" s="14" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>program</t>
         </is>
       </c>
       <c r="D213" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream quote</t>
+          <t>kiwoom stream program</t>
         </is>
       </c>
       <c r="E213" s="14" t="inlineStr">
         <is>
-          <t>주식체결 실시간 (0B)</t>
+          <t>종목프로그램매매 실시간 (0w)</t>
         </is>
       </c>
       <c r="F213" s="15" t="inlineStr"/>
@@ -9496,17 +9497,17 @@
       </c>
       <c r="C214" s="14" t="inlineStr">
         <is>
-          <t>sector-change</t>
+          <t>quote</t>
         </is>
       </c>
       <c r="D214" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream sector-change</t>
+          <t>kiwoom stream quote</t>
         </is>
       </c>
       <c r="E214" s="14" t="inlineStr">
         <is>
-          <t>업종등락 실시간 (0U)</t>
+          <t>주식체결 실시간 (0B)</t>
         </is>
       </c>
       <c r="F214" s="15" t="inlineStr"/>
@@ -9534,17 +9535,17 @@
       </c>
       <c r="C215" s="14" t="inlineStr">
         <is>
-          <t>sector-index</t>
+          <t>sector-change</t>
         </is>
       </c>
       <c r="D215" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream sector-index</t>
+          <t>kiwoom stream sector-change</t>
         </is>
       </c>
       <c r="E215" s="14" t="inlineStr">
         <is>
-          <t>업종지수 실시간 (0J)</t>
+          <t>업종등락 실시간 (0U)</t>
         </is>
       </c>
       <c r="F215" s="15" t="inlineStr"/>
@@ -9572,17 +9573,17 @@
       </c>
       <c r="C216" s="14" t="inlineStr">
         <is>
-          <t>stock-info</t>
+          <t>sector-index</t>
         </is>
       </c>
       <c r="D216" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream stock-info</t>
+          <t>kiwoom stream sector-index</t>
         </is>
       </c>
       <c r="E216" s="14" t="inlineStr">
         <is>
-          <t>주식종목정보 실시간 (0g)</t>
+          <t>업종지수 실시간 (0J)</t>
         </is>
       </c>
       <c r="F216" s="15" t="inlineStr"/>
@@ -9610,17 +9611,17 @@
       </c>
       <c r="C217" s="14" t="inlineStr">
         <is>
-          <t>trader</t>
+          <t>stock-info</t>
         </is>
       </c>
       <c r="D217" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream trader</t>
+          <t>kiwoom stream stock-info</t>
         </is>
       </c>
       <c r="E217" s="14" t="inlineStr">
         <is>
-          <t>주식당일거래원 실시간 (0F)</t>
+          <t>주식종목정보 실시간 (0g)</t>
         </is>
       </c>
       <c r="F217" s="15" t="inlineStr"/>
@@ -9648,28 +9649,28 @@
       </c>
       <c r="C218" s="14" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>trader</t>
         </is>
       </c>
       <c r="D218" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream types</t>
+          <t>kiwoom stream trader</t>
         </is>
       </c>
       <c r="E218" s="14" t="inlineStr">
         <is>
-          <t>사용 가능한 실시간 타입 코드 목록</t>
+          <t>주식당일거래원 실시간 (0F)</t>
         </is>
       </c>
       <c r="F218" s="15" t="inlineStr"/>
       <c r="G218" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H218" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--raw (JSON 원본 출력)</t>
         </is>
       </c>
     </row>
@@ -9686,64 +9687,102 @@
       </c>
       <c r="C219" s="14" t="inlineStr">
         <is>
-          <t>vi</t>
+          <t>types</t>
         </is>
       </c>
       <c r="D219" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream vi</t>
+          <t>kiwoom stream types</t>
         </is>
       </c>
       <c r="E219" s="14" t="inlineStr">
         <is>
-          <t>VI발동/해제 실시간 (1h)</t>
+          <t>사용 가능한 실시간 타입 코드 목록</t>
         </is>
       </c>
       <c r="F219" s="15" t="inlineStr"/>
       <c r="G219" s="14" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H219" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="14" t="inlineStr">
+        <is>
+          <t>stream</t>
+        </is>
+      </c>
+      <c r="B220" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C220" s="14" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="D220" s="14" t="inlineStr">
+        <is>
+          <t>kiwoom stream vi</t>
+        </is>
+      </c>
+      <c r="E220" s="14" t="inlineStr">
+        <is>
+          <t>VI발동/해제 실시간 (1h)</t>
+        </is>
+      </c>
+      <c r="F220" s="15" t="inlineStr"/>
+      <c r="G220" s="14" t="inlineStr">
+        <is>
           <t>CODES (복수) (필수)</t>
         </is>
       </c>
-      <c r="H219" s="14" t="inlineStr">
+      <c r="H220" s="14" t="inlineStr">
         <is>
           <t>--raw (JSON 원본 출력)</t>
         </is>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="6" t="inlineStr">
+    <row r="221">
+      <c r="A221" s="6" t="inlineStr">
         <is>
           <t>watch</t>
         </is>
       </c>
-      <c r="B220" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C220" s="6" t="inlineStr">
+      <c r="B221" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C221" s="6" t="inlineStr">
         <is>
           <t>watch</t>
         </is>
       </c>
-      <c r="D220" s="6" t="inlineStr">
+      <c r="D221" s="6" t="inlineStr">
         <is>
           <t>kiwoom watch</t>
         </is>
       </c>
-      <c r="E220" s="6" t="inlineStr">
+      <c r="E221" s="6" t="inlineStr">
         <is>
           <t>실시간 종목 모니터링 (TUI 대시보드)</t>
         </is>
       </c>
-      <c r="F220" s="7" t="inlineStr"/>
-      <c r="G220" s="6" t="inlineStr">
+      <c r="F221" s="7" t="inlineStr"/>
+      <c r="G221" s="6" t="inlineStr">
         <is>
           <t>CODES (복수) (필수)</t>
         </is>
       </c>
-      <c r="H220" s="6" t="inlineStr">
+      <c r="H221" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9776,6 +9815,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
@@ -9845,7 +9885,7 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
@@ -9950,7 +9990,7 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README and Excel: remove stock list, update search description
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$220</definedName>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H221"/>
+  <dimension ref="A1:H220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8573,46 +8573,50 @@
       </c>
       <c r="H190" s="12" t="inlineStr">
         <is>
-          <t>--market [kospi, kosdaq, k-otc, konex, etf, elw] 기본:kospi (시장구분 (kospi/kosdaq/k-otc/konex/etf/elw))</t>
+          <t>--market [all, kospi, kosdaq, k-otc, konex, etf, elw] 기본:all (시장구분 (all/kospi/kosdaq/k-otc/konex/etf/elw))</t>
         </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr">
+      <c r="A191" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>list</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>kiwoom stock list</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>KRX 전체 상장종목 리스트 (pykrx)</t>
-        </is>
-      </c>
-      <c r="G191" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>--market [all, kospi, kosdaq, konex] 기본:all (시장구분)
---search (종목명/코드 검색 키워드)
---refresh (캐시 무시하고 새로 조회)</t>
+      <c r="B191" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C191" s="12" t="inlineStr">
+        <is>
+          <t>short</t>
+        </is>
+      </c>
+      <c r="D191" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock short</t>
+        </is>
+      </c>
+      <c r="E191" s="12" t="inlineStr">
+        <is>
+          <t>공매도 추이 조회</t>
+        </is>
+      </c>
+      <c r="F191" s="13" t="inlineStr">
+        <is>
+          <t>ka10014</t>
+        </is>
+      </c>
+      <c r="G191" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H191" s="12" t="inlineStr">
+        <is>
+          <t>--from (시작일자 (YYYYMMDD, 기본=30일전))
+--to (종료일자 (YYYYMMDD, 기본=오늘))</t>
         </is>
       </c>
     </row>
@@ -8629,22 +8633,22 @@
       </c>
       <c r="C192" s="12" t="inlineStr">
         <is>
-          <t>short</t>
+          <t>tick-strength</t>
         </is>
       </c>
       <c r="D192" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock short</t>
+          <t>kiwoom stock tick-strength</t>
         </is>
       </c>
       <c r="E192" s="12" t="inlineStr">
         <is>
-          <t>공매도 추이 조회</t>
+          <t>체결강도추이 시간별</t>
         </is>
       </c>
       <c r="F192" s="13" t="inlineStr">
         <is>
-          <t>ka10014</t>
+          <t>ka10046</t>
         </is>
       </c>
       <c r="G192" s="12" t="inlineStr">
@@ -8654,8 +8658,7 @@
       </c>
       <c r="H192" s="12" t="inlineStr">
         <is>
-          <t>--from (시작일자 (YYYYMMDD, 기본=30일전))
---to (종료일자 (YYYYMMDD, 기본=오늘))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -8672,22 +8675,22 @@
       </c>
       <c r="C193" s="12" t="inlineStr">
         <is>
-          <t>tick-strength</t>
+          <t>timeprice</t>
         </is>
       </c>
       <c r="D193" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock tick-strength</t>
+          <t>kiwoom stock timeprice</t>
         </is>
       </c>
       <c r="E193" s="12" t="inlineStr">
         <is>
-          <t>체결강도추이 시간별</t>
+          <t>시분 시세 조회</t>
         </is>
       </c>
       <c r="F193" s="13" t="inlineStr">
         <is>
-          <t>ka10046</t>
+          <t>ka10006</t>
         </is>
       </c>
       <c r="G193" s="12" t="inlineStr">
@@ -8714,22 +8717,22 @@
       </c>
       <c r="C194" s="12" t="inlineStr">
         <is>
-          <t>timeprice</t>
+          <t>today-exec</t>
         </is>
       </c>
       <c r="D194" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock timeprice</t>
+          <t>kiwoom stock today-exec</t>
         </is>
       </c>
       <c r="E194" s="12" t="inlineStr">
         <is>
-          <t>시분 시세 조회</t>
+          <t>당일/전일 체결 조회</t>
         </is>
       </c>
       <c r="F194" s="13" t="inlineStr">
         <is>
-          <t>ka10006</t>
+          <t>ka10084</t>
         </is>
       </c>
       <c r="G194" s="12" t="inlineStr">
@@ -8738,48 +8741,6 @@
         </is>
       </c>
       <c r="H194" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B195" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C195" s="12" t="inlineStr">
-        <is>
-          <t>today-exec</t>
-        </is>
-      </c>
-      <c r="D195" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock today-exec</t>
-        </is>
-      </c>
-      <c r="E195" s="12" t="inlineStr">
-        <is>
-          <t>당일/전일 체결 조회</t>
-        </is>
-      </c>
-      <c r="F195" s="13" t="inlineStr">
-        <is>
-          <t>ka10084</t>
-        </is>
-      </c>
-      <c r="G195" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H195" s="12" t="inlineStr">
         <is>
           <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))
 --mode [0, 1] (틱/분 (0=틱, 1=분))
@@ -8787,6 +8748,48 @@
         </is>
       </c>
     </row>
+    <row r="195">
+      <c r="A195" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B195" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C195" s="12" t="inlineStr">
+        <is>
+          <t>today-volume</t>
+        </is>
+      </c>
+      <c r="D195" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock today-volume</t>
+        </is>
+      </c>
+      <c r="E195" s="12" t="inlineStr">
+        <is>
+          <t>당일/전일 체결량 조회</t>
+        </is>
+      </c>
+      <c r="F195" s="13" t="inlineStr">
+        <is>
+          <t>ka10055</t>
+        </is>
+      </c>
+      <c r="G195" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H195" s="12" t="inlineStr">
+        <is>
+          <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))</t>
+        </is>
+      </c>
+    </row>
     <row r="196">
       <c r="A196" s="12" t="inlineStr">
         <is>
@@ -8800,22 +8803,22 @@
       </c>
       <c r="C196" s="12" t="inlineStr">
         <is>
-          <t>today-volume</t>
+          <t>trader</t>
         </is>
       </c>
       <c r="D196" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock today-volume</t>
+          <t>kiwoom stock trader</t>
         </is>
       </c>
       <c r="E196" s="12" t="inlineStr">
         <is>
-          <t>당일/전일 체결량 조회</t>
+          <t>거래원 조회</t>
         </is>
       </c>
       <c r="F196" s="13" t="inlineStr">
         <is>
-          <t>ka10055</t>
+          <t>ka10002</t>
         </is>
       </c>
       <c r="G196" s="12" t="inlineStr">
@@ -8825,7 +8828,7 @@
       </c>
       <c r="H196" s="12" t="inlineStr">
         <is>
-          <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -8842,27 +8845,27 @@
       </c>
       <c r="C197" s="12" t="inlineStr">
         <is>
-          <t>trader</t>
+          <t>watchlist</t>
         </is>
       </c>
       <c r="D197" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock trader</t>
+          <t>kiwoom stock watchlist</t>
         </is>
       </c>
       <c r="E197" s="12" t="inlineStr">
         <is>
-          <t>거래원 조회</t>
+          <t>관심종목정보 조회 (코드를 |로 구분, 예: 005930|000660)</t>
         </is>
       </c>
       <c r="F197" s="13" t="inlineStr">
         <is>
-          <t>ka10002</t>
+          <t>ka10095</t>
         </is>
       </c>
       <c r="G197" s="12" t="inlineStr">
         <is>
-          <t>CODE (필수)</t>
+          <t>CODES (필수)</t>
         </is>
       </c>
       <c r="H197" s="12" t="inlineStr">
@@ -8872,44 +8875,40 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B198" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C198" s="12" t="inlineStr">
-        <is>
-          <t>watchlist</t>
-        </is>
-      </c>
-      <c r="D198" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock watchlist</t>
-        </is>
-      </c>
-      <c r="E198" s="12" t="inlineStr">
-        <is>
-          <t>관심종목정보 조회 (코드를 |로 구분, 예: 005930|000660)</t>
-        </is>
-      </c>
-      <c r="F198" s="13" t="inlineStr">
-        <is>
-          <t>ka10095</t>
-        </is>
-      </c>
-      <c r="G198" s="12" t="inlineStr">
-        <is>
-          <t>CODES (필수)</t>
-        </is>
-      </c>
-      <c r="H198" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="A198" s="14" t="inlineStr">
+        <is>
+          <t>stream</t>
+        </is>
+      </c>
+      <c r="B198" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C198" s="14" t="inlineStr">
+        <is>
+          <t>after-hours</t>
+        </is>
+      </c>
+      <c r="D198" s="14" t="inlineStr">
+        <is>
+          <t>kiwoom stream after-hours</t>
+        </is>
+      </c>
+      <c r="E198" s="14" t="inlineStr">
+        <is>
+          <t>주식시간외호가 실시간 (0E)</t>
+        </is>
+      </c>
+      <c r="F198" s="15" t="inlineStr"/>
+      <c r="G198" s="14" t="inlineStr">
+        <is>
+          <t>CODES (복수) (필수)</t>
+        </is>
+      </c>
+      <c r="H198" s="14" t="inlineStr">
+        <is>
+          <t>--raw (JSON 원본 출력)</t>
         </is>
       </c>
     </row>
@@ -8926,23 +8925,23 @@
       </c>
       <c r="C199" s="14" t="inlineStr">
         <is>
-          <t>after-hours</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="D199" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream after-hours</t>
+          <t>kiwoom stream balance</t>
         </is>
       </c>
       <c r="E199" s="14" t="inlineStr">
         <is>
-          <t>주식시간외호가 실시간 (0E)</t>
+          <t>잔고 실시간 (04)</t>
         </is>
       </c>
       <c r="F199" s="15" t="inlineStr"/>
       <c r="G199" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H199" s="14" t="inlineStr">
@@ -8964,23 +8963,23 @@
       </c>
       <c r="C200" s="14" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>best-bid</t>
         </is>
       </c>
       <c r="D200" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream balance</t>
+          <t>kiwoom stream best-bid</t>
         </is>
       </c>
       <c r="E200" s="14" t="inlineStr">
         <is>
-          <t>잔고 실시간 (04)</t>
+          <t>주식우선호가 실시간 (0C)</t>
         </is>
       </c>
       <c r="F200" s="15" t="inlineStr"/>
       <c r="G200" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H200" s="14" t="inlineStr">
@@ -9002,23 +9001,24 @@
       </c>
       <c r="C201" s="14" t="inlineStr">
         <is>
-          <t>best-bid</t>
+          <t>custom</t>
         </is>
       </c>
       <c r="D201" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream best-bid</t>
+          <t>kiwoom stream custom</t>
         </is>
       </c>
       <c r="E201" s="14" t="inlineStr">
         <is>
-          <t>주식우선호가 실시간 (0C)</t>
+          <t>커스텀 실시간 타입으로 스트리밍</t>
         </is>
       </c>
       <c r="F201" s="15" t="inlineStr"/>
       <c r="G201" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>TYPE_CODES (필수)
+CODES (복수) (선택)</t>
         </is>
       </c>
       <c r="H201" s="14" t="inlineStr">
@@ -9040,24 +9040,23 @@
       </c>
       <c r="C202" s="14" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>elw-indicator</t>
         </is>
       </c>
       <c r="D202" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream custom</t>
+          <t>kiwoom stream elw-indicator</t>
         </is>
       </c>
       <c r="E202" s="14" t="inlineStr">
         <is>
-          <t>커스텀 실시간 타입으로 스트리밍</t>
+          <t>ELW 지표 실시간 (0u)</t>
         </is>
       </c>
       <c r="F202" s="15" t="inlineStr"/>
       <c r="G202" s="14" t="inlineStr">
         <is>
-          <t>TYPE_CODES (필수)
-CODES (복수) (선택)</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H202" s="14" t="inlineStr">
@@ -9079,17 +9078,17 @@
       </c>
       <c r="C203" s="14" t="inlineStr">
         <is>
-          <t>elw-indicator</t>
+          <t>elw-theory</t>
         </is>
       </c>
       <c r="D203" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream elw-indicator</t>
+          <t>kiwoom stream elw-theory</t>
         </is>
       </c>
       <c r="E203" s="14" t="inlineStr">
         <is>
-          <t>ELW 지표 실시간 (0u)</t>
+          <t>ELW 이론가 실시간 (0m)</t>
         </is>
       </c>
       <c r="F203" s="15" t="inlineStr"/>
@@ -9117,17 +9116,17 @@
       </c>
       <c r="C204" s="14" t="inlineStr">
         <is>
-          <t>elw-theory</t>
+          <t>etf-nav</t>
         </is>
       </c>
       <c r="D204" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream elw-theory</t>
+          <t>kiwoom stream etf-nav</t>
         </is>
       </c>
       <c r="E204" s="14" t="inlineStr">
         <is>
-          <t>ELW 이론가 실시간 (0m)</t>
+          <t>ETF NAV 실시간 (0G)</t>
         </is>
       </c>
       <c r="F204" s="15" t="inlineStr"/>
@@ -9155,17 +9154,17 @@
       </c>
       <c r="C205" s="14" t="inlineStr">
         <is>
-          <t>etf-nav</t>
+          <t>expected</t>
         </is>
       </c>
       <c r="D205" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream etf-nav</t>
+          <t>kiwoom stream expected</t>
         </is>
       </c>
       <c r="E205" s="14" t="inlineStr">
         <is>
-          <t>ETF NAV 실시간 (0G)</t>
+          <t>주식예상체결 실시간 (0H)</t>
         </is>
       </c>
       <c r="F205" s="15" t="inlineStr"/>
@@ -9193,17 +9192,17 @@
       </c>
       <c r="C206" s="14" t="inlineStr">
         <is>
-          <t>expected</t>
+          <t>gold</t>
         </is>
       </c>
       <c r="D206" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream expected</t>
+          <t>kiwoom stream gold</t>
         </is>
       </c>
       <c r="E206" s="14" t="inlineStr">
         <is>
-          <t>주식예상체결 실시간 (0H)</t>
+          <t>국제금환산가격 실시간 (0I)</t>
         </is>
       </c>
       <c r="F206" s="15" t="inlineStr"/>
@@ -9231,23 +9230,23 @@
       </c>
       <c r="C207" s="14" t="inlineStr">
         <is>
-          <t>gold</t>
+          <t>market-time</t>
         </is>
       </c>
       <c r="D207" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream gold</t>
+          <t>kiwoom stream market-time</t>
         </is>
       </c>
       <c r="E207" s="14" t="inlineStr">
         <is>
-          <t>국제금환산가격 실시간 (0I)</t>
+          <t>장시작시간 실시간 (0s)</t>
         </is>
       </c>
       <c r="F207" s="15" t="inlineStr"/>
       <c r="G207" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H207" s="14" t="inlineStr">
@@ -9269,23 +9268,23 @@
       </c>
       <c r="C208" s="14" t="inlineStr">
         <is>
-          <t>market-time</t>
+          <t>multi</t>
         </is>
       </c>
       <c r="D208" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream market-time</t>
+          <t>kiwoom stream multi</t>
         </is>
       </c>
       <c r="E208" s="14" t="inlineStr">
         <is>
-          <t>장시작시간 실시간 (0s)</t>
+          <t>주식체결+호가잔량 동시 스트리밍 (0B+0D)</t>
         </is>
       </c>
       <c r="F208" s="15" t="inlineStr"/>
       <c r="G208" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H208" s="14" t="inlineStr">
@@ -9307,23 +9306,23 @@
       </c>
       <c r="C209" s="14" t="inlineStr">
         <is>
-          <t>multi</t>
+          <t>order</t>
         </is>
       </c>
       <c r="D209" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream multi</t>
+          <t>kiwoom stream order</t>
         </is>
       </c>
       <c r="E209" s="14" t="inlineStr">
         <is>
-          <t>주식체결+호가잔량 동시 스트리밍 (0B+0D)</t>
+          <t>주문체결 실시간 (00)</t>
         </is>
       </c>
       <c r="F209" s="15" t="inlineStr"/>
       <c r="G209" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H209" s="14" t="inlineStr">
@@ -9345,23 +9344,23 @@
       </c>
       <c r="C210" s="14" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>orderbook</t>
         </is>
       </c>
       <c r="D210" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream order</t>
+          <t>kiwoom stream orderbook</t>
         </is>
       </c>
       <c r="E210" s="14" t="inlineStr">
         <is>
-          <t>주문체결 실시간 (00)</t>
+          <t>주식호가잔량 실시간 (0D)</t>
         </is>
       </c>
       <c r="F210" s="15" t="inlineStr"/>
       <c r="G210" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H210" s="14" t="inlineStr">
@@ -9383,17 +9382,17 @@
       </c>
       <c r="C211" s="14" t="inlineStr">
         <is>
-          <t>orderbook</t>
+          <t>price</t>
         </is>
       </c>
       <c r="D211" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream orderbook</t>
+          <t>kiwoom stream price</t>
         </is>
       </c>
       <c r="E211" s="14" t="inlineStr">
         <is>
-          <t>주식호가잔량 실시간 (0D)</t>
+          <t>주식기세 실시간 (0A)</t>
         </is>
       </c>
       <c r="F211" s="15" t="inlineStr"/>
@@ -9421,17 +9420,17 @@
       </c>
       <c r="C212" s="14" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>program</t>
         </is>
       </c>
       <c r="D212" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream price</t>
+          <t>kiwoom stream program</t>
         </is>
       </c>
       <c r="E212" s="14" t="inlineStr">
         <is>
-          <t>주식기세 실시간 (0A)</t>
+          <t>종목프로그램매매 실시간 (0w)</t>
         </is>
       </c>
       <c r="F212" s="15" t="inlineStr"/>
@@ -9459,17 +9458,17 @@
       </c>
       <c r="C213" s="14" t="inlineStr">
         <is>
-          <t>program</t>
+          <t>quote</t>
         </is>
       </c>
       <c r="D213" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream program</t>
+          <t>kiwoom stream quote</t>
         </is>
       </c>
       <c r="E213" s="14" t="inlineStr">
         <is>
-          <t>종목프로그램매매 실시간 (0w)</t>
+          <t>주식체결 실시간 (0B)</t>
         </is>
       </c>
       <c r="F213" s="15" t="inlineStr"/>
@@ -9497,17 +9496,17 @@
       </c>
       <c r="C214" s="14" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>sector-change</t>
         </is>
       </c>
       <c r="D214" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream quote</t>
+          <t>kiwoom stream sector-change</t>
         </is>
       </c>
       <c r="E214" s="14" t="inlineStr">
         <is>
-          <t>주식체결 실시간 (0B)</t>
+          <t>업종등락 실시간 (0U)</t>
         </is>
       </c>
       <c r="F214" s="15" t="inlineStr"/>
@@ -9535,17 +9534,17 @@
       </c>
       <c r="C215" s="14" t="inlineStr">
         <is>
-          <t>sector-change</t>
+          <t>sector-index</t>
         </is>
       </c>
       <c r="D215" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream sector-change</t>
+          <t>kiwoom stream sector-index</t>
         </is>
       </c>
       <c r="E215" s="14" t="inlineStr">
         <is>
-          <t>업종등락 실시간 (0U)</t>
+          <t>업종지수 실시간 (0J)</t>
         </is>
       </c>
       <c r="F215" s="15" t="inlineStr"/>
@@ -9573,17 +9572,17 @@
       </c>
       <c r="C216" s="14" t="inlineStr">
         <is>
-          <t>sector-index</t>
+          <t>stock-info</t>
         </is>
       </c>
       <c r="D216" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream sector-index</t>
+          <t>kiwoom stream stock-info</t>
         </is>
       </c>
       <c r="E216" s="14" t="inlineStr">
         <is>
-          <t>업종지수 실시간 (0J)</t>
+          <t>주식종목정보 실시간 (0g)</t>
         </is>
       </c>
       <c r="F216" s="15" t="inlineStr"/>
@@ -9611,17 +9610,17 @@
       </c>
       <c r="C217" s="14" t="inlineStr">
         <is>
-          <t>stock-info</t>
+          <t>trader</t>
         </is>
       </c>
       <c r="D217" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream stock-info</t>
+          <t>kiwoom stream trader</t>
         </is>
       </c>
       <c r="E217" s="14" t="inlineStr">
         <is>
-          <t>주식종목정보 실시간 (0g)</t>
+          <t>주식당일거래원 실시간 (0F)</t>
         </is>
       </c>
       <c r="F217" s="15" t="inlineStr"/>
@@ -9649,28 +9648,28 @@
       </c>
       <c r="C218" s="14" t="inlineStr">
         <is>
-          <t>trader</t>
+          <t>types</t>
         </is>
       </c>
       <c r="D218" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream trader</t>
+          <t>kiwoom stream types</t>
         </is>
       </c>
       <c r="E218" s="14" t="inlineStr">
         <is>
-          <t>주식당일거래원 실시간 (0F)</t>
+          <t>사용 가능한 실시간 타입 코드 목록</t>
         </is>
       </c>
       <c r="F218" s="15" t="inlineStr"/>
       <c r="G218" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H218" s="14" t="inlineStr">
         <is>
-          <t>--raw (JSON 원본 출력)</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -9687,102 +9686,64 @@
       </c>
       <c r="C219" s="14" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>vi</t>
         </is>
       </c>
       <c r="D219" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream types</t>
+          <t>kiwoom stream vi</t>
         </is>
       </c>
       <c r="E219" s="14" t="inlineStr">
         <is>
-          <t>사용 가능한 실시간 타입 코드 목록</t>
+          <t>VI발동/해제 실시간 (1h)</t>
         </is>
       </c>
       <c r="F219" s="15" t="inlineStr"/>
       <c r="G219" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H219" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--raw (JSON 원본 출력)</t>
         </is>
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="14" t="inlineStr">
-        <is>
-          <t>stream</t>
-        </is>
-      </c>
-      <c r="B220" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C220" s="14" t="inlineStr">
-        <is>
-          <t>vi</t>
-        </is>
-      </c>
-      <c r="D220" s="14" t="inlineStr">
-        <is>
-          <t>kiwoom stream vi</t>
-        </is>
-      </c>
-      <c r="E220" s="14" t="inlineStr">
-        <is>
-          <t>VI발동/해제 실시간 (1h)</t>
-        </is>
-      </c>
-      <c r="F220" s="15" t="inlineStr"/>
-      <c r="G220" s="14" t="inlineStr">
+      <c r="A220" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="B220" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C220" s="6" t="inlineStr">
+        <is>
+          <t>watch</t>
+        </is>
+      </c>
+      <c r="D220" s="6" t="inlineStr">
+        <is>
+          <t>kiwoom watch</t>
+        </is>
+      </c>
+      <c r="E220" s="6" t="inlineStr">
+        <is>
+          <t>실시간 종목 모니터링 (TUI 대시보드)</t>
+        </is>
+      </c>
+      <c r="F220" s="7" t="inlineStr"/>
+      <c r="G220" s="6" t="inlineStr">
         <is>
           <t>CODES (복수) (필수)</t>
         </is>
       </c>
-      <c r="H220" s="14" t="inlineStr">
-        <is>
-          <t>--raw (JSON 원본 출력)</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="6" t="inlineStr">
-        <is>
-          <t>watch</t>
-        </is>
-      </c>
-      <c r="B221" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C221" s="6" t="inlineStr">
-        <is>
-          <t>watch</t>
-        </is>
-      </c>
-      <c r="D221" s="6" t="inlineStr">
-        <is>
-          <t>kiwoom watch</t>
-        </is>
-      </c>
-      <c r="E221" s="6" t="inlineStr">
-        <is>
-          <t>실시간 종목 모니터링 (TUI 대시보드)</t>
-        </is>
-      </c>
-      <c r="F221" s="7" t="inlineStr"/>
-      <c r="G221" s="6" t="inlineStr">
-        <is>
-          <t>CODES (복수) (필수)</t>
-        </is>
-      </c>
-      <c r="H221" s="6" t="inlineStr">
+      <c r="H220" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9815,7 +9776,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
@@ -9885,7 +9845,7 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
@@ -9990,7 +9950,7 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add config set command, update README and Excel (222 commands)
Bump version to 0.6.2

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1940,23 +1940,23 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>domain</t>
+          <t>profiles</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>kiwoom config domain</t>
+          <t>kiwoom config profiles</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>도메인 변경 (prod/mock)</t>
+          <t>등록된 프로필 목록</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>DOMAIN (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -1978,23 +1978,24 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>profiles</t>
+          <t>set</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>kiwoom config profiles</t>
+          <t>kiwoom config set</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>등록된 프로필 목록</t>
+          <t>프로필 설정 변경</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr"/>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>KEY (필수)
+VALUE (필수)</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -9934,7 +9935,7 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>인증 (토큰)</t>
+          <t>인증</t>
         </is>
       </c>
     </row>
@@ -9949,7 +9950,7 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Raw API 호출</t>
+          <t>Raw API</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate Excel (222 commands)
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$223</definedName>
@@ -2041,8 +2041,8 @@
           <t>--profile 기본:default (프로필 이름)
 --appkey (키움 API App Key)
 --secretkey (키움 API Secret Key)
---domain [prod, mock] 기본:mock (도메인 (prod: 실거래, mock: 모의투자))
---account (기본 계좌번호)</t>
+--domain [prod, mock] 기본:mock (도메인)
+--account (계좌번호)</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5519,7 @@
 --type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (조건부가격 (스톱지정가 등))
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5564,7 +5564,7 @@
         <is>
           <t>--qty (취소수량 (0=전량취소))
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5606,7 +5606,7 @@
       </c>
       <c r="H123" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5649,7 +5649,7 @@
       <c r="H124" s="10" t="inlineStr">
         <is>
           <t>--exchange [K] 기본:K (거래소 (K=KRX))
---confirm *필수 (조회 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5694,7 +5694,7 @@
           <t>--exchange [K] 기본:K (거래소 (K=KRX))
 --cont-yn (연속조회여부)
 --next-key (연속조회키)
---confirm *필수 (조회 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="H126" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5783,7 +5783,7 @@
 --type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (조건부가격)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
         <is>
           <t>--qty (취소수량 (0=전량취소))
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5875,7 +5875,7 @@
         <is>
           <t>--exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (정정 조건부가격)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5922,7 +5922,7 @@
 --type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (조건부가격)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="H131" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6010,7 +6010,7 @@
           <t>--price (주문가격 (시장가 주문시 생략))
 --type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
         <is>
           <t>--qty (취소수량 (0=전량취소))
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="H134" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="H136" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6223,7 @@
       </c>
       <c r="H137" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6269,7 +6269,7 @@
       <c r="H138" s="10" t="inlineStr">
         <is>
           <t>--exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -6311,7 +6311,7 @@
       </c>
       <c r="H139" s="10" t="inlineStr">
         <is>
-          <t>--confirm *필수 (조회 확인 (필수))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
           <t>--price (주문가격 (시장가 주문시 생략))
 --type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -6404,7 +6404,7 @@
         <is>
           <t>--exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (정정 조건부가격)
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>
@@ -6451,7 +6451,7 @@
 --type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (조건부가격 (스톱지정가 등))
---confirm *필수 (주문 확인 (필수))</t>
+--confirm (확인 프롬프트 없이 주문 실행)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: bump version to 2.2.0
- KIWOOM_TOKEN 환경변수 지원 (키체인 접근 불가 환경용, 키체인 토큰보다 우선)
- config setup에서 토큰 저장 방식 선택 (keychain/env)
- CHANGELOG v2.2.0 항목 추가, Excel 명령어 레퍼런스 재생성

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1944,7 +1944,7 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>접근토큰 발급 (비밀번호 확인 후 암호화된 인증정보 사용)</t>
+          <t>접근토큰 발급</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>접근토큰 폐기 (비밀번호 확인 필요)</t>
+          <t>접근토큰 폐기</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr"/>
@@ -2150,7 +2150,8 @@
 --appkey (키움 API App Key)
 --secretkey (키움 API Secret Key)
 --domain [prod, mock] 기본:mock (도메인)
---account (계좌번호)</t>
+--account (계좌번호)
+--token-storage [keychain, env] 기본:keychain (접근토큰 저장 방식)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release: bump version to 2.4.0
- order: --dry-run (전송 없이 body 확인), order validate 사전점검,
  --client-order-id 멱등키, json/csv 모드 CONFIRMATION_REQUIRED (프롬프트 제거)
- --confirm에 --yes 별칭 추가
- fix: US stock info 거래소 자동판별 (usa10100 stex_tp)
- fix: 키체인 접근 불가 환경에서 KIWOOM_TOKEN 안내

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -11,7 +11,7 @@
     <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$226</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$227</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H226"/>
+  <dimension ref="A1:H227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5625,7 +5625,9 @@
 --type [after-hours, best, best-fok, best-ioc, conditional, first, fok, ioc, limit, loc, market, market-fok, market-ioc, mid, mid-fok, mid-ioc, moc, pre-market, single, stop, stop-limit, twap, twap-limit, vwap, vwap-limit] 기본:market (주문유형)
 --exchange [KRX, NXT, SOR, nasdaq, nyse, amex] (거래소 (기본: 국내 KRX / 미국 자동판별))
 --cond-price (조건부가격 (국내 전용))
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5668,9 @@
         <is>
           <t>--qty (취소수량 (0=전량취소, 미국은 전량취소만 지원))
 --exchange [KRX, NXT, SOR, nasdaq, nyse, amex] (거래소 (기본: 국내 KRX / 미국 자동판별))
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6499,7 +6503,9 @@
           <t>--exchange [KRX, NXT, SOR, nasdaq, nyse, amex] (거래소 (기본: 국내 KRX / 미국 자동판별))
 --cond-price (정정 조건부가격 (국내 전용))
 --stop (STOP가격 (미국 정정 전용))
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6543,49 +6549,51 @@
 --exchange [KRX, NXT, SOR, nasdaq, nyse, amex] (거래소 (기본: 국내 KRX / 미국 자동판별))
 --cond-price (조건부가격 (국내 전용))
 --stop (STOP가격 (미국 stop/stop-limit 전용))
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B146" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C146" s="12" t="inlineStr">
-        <is>
-          <t>after-hours</t>
-        </is>
-      </c>
-      <c r="D146" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock after-hours</t>
-        </is>
-      </c>
-      <c r="E146" s="12" t="inlineStr">
-        <is>
-          <t>시간외단일가 조회</t>
-        </is>
-      </c>
-      <c r="F146" s="13" t="inlineStr">
-        <is>
-          <t>ka10087</t>
-        </is>
-      </c>
-      <c r="G146" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H146" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="A146" s="10" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C146" s="10" t="inlineStr">
+        <is>
+          <t>validate</t>
+        </is>
+      </c>
+      <c r="D146" s="10" t="inlineStr">
+        <is>
+          <t>kiwoom order validate</t>
+        </is>
+      </c>
+      <c r="E146" s="10" t="inlineStr">
+        <is>
+          <t>주문 사전점검 — 주문을 전송하지 않는 read-only 프리플라이트</t>
+        </is>
+      </c>
+      <c r="F146" s="11" t="inlineStr"/>
+      <c r="G146" s="10" t="inlineStr">
+        <is>
+          <t>SIDE (필수)
+CODE (필수)
+QTY (필수)</t>
+        </is>
+      </c>
+      <c r="H146" s="10" t="inlineStr">
+        <is>
+          <t>--price (주문가격 (생략 시 현재가로 예상비용 계산))
+--type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
+--exchange [KRX, NXT] 기본:KRX (거래소)</t>
         </is>
       </c>
     </row>
@@ -6597,35 +6605,77 @@
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C147" s="12" t="inlineStr">
+        <is>
+          <t>after-hours</t>
+        </is>
+      </c>
+      <c r="D147" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock after-hours</t>
+        </is>
+      </c>
+      <c r="E147" s="12" t="inlineStr">
+        <is>
+          <t>시간외단일가 조회</t>
+        </is>
+      </c>
+      <c r="F147" s="13" t="inlineStr">
+        <is>
+          <t>ka10087</t>
+        </is>
+      </c>
+      <c r="G147" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H147" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C147" s="12" t="inlineStr">
+      <c r="C148" s="12" t="inlineStr">
         <is>
           <t>broker-stock</t>
         </is>
       </c>
-      <c r="D147" s="12" t="inlineStr">
+      <c r="D148" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis broker-stock</t>
         </is>
       </c>
-      <c r="E147" s="12" t="inlineStr">
+      <c r="E148" s="12" t="inlineStr">
         <is>
           <t>증권사별종목매매동향 조회</t>
         </is>
       </c>
-      <c r="F147" s="13" t="inlineStr">
+      <c r="F148" s="13" t="inlineStr">
         <is>
           <t>ka10078</t>
         </is>
       </c>
-      <c r="G147" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H147" s="12" t="inlineStr">
+      <c r="G148" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H148" s="12" t="inlineStr">
         <is>
           <t>--broker *필수 (회원사코드)
 --code *필수 (종목코드)
@@ -6634,48 +6684,6 @@
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B148" s="12" t="inlineStr">
-        <is>
-          <t>analysis</t>
-        </is>
-      </c>
-      <c r="C148" s="12" t="inlineStr">
-        <is>
-          <t>daily-detail</t>
-        </is>
-      </c>
-      <c r="D148" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock analysis daily-detail</t>
-        </is>
-      </c>
-      <c r="E148" s="12" t="inlineStr">
-        <is>
-          <t>일별거래상세 조회</t>
-        </is>
-      </c>
-      <c r="F148" s="13" t="inlineStr">
-        <is>
-          <t>ka10015</t>
-        </is>
-      </c>
-      <c r="G148" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H148" s="12" t="inlineStr">
-        <is>
-          <t>--from *필수 (시작일자 (YYYYMMDD))</t>
-        </is>
-      </c>
-    </row>
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
@@ -6689,30 +6697,72 @@
       </c>
       <c r="C149" s="12" t="inlineStr">
         <is>
+          <t>daily-detail</t>
+        </is>
+      </c>
+      <c r="D149" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock analysis daily-detail</t>
+        </is>
+      </c>
+      <c r="E149" s="12" t="inlineStr">
+        <is>
+          <t>일별거래상세 조회</t>
+        </is>
+      </c>
+      <c r="F149" s="13" t="inlineStr">
+        <is>
+          <t>ka10015</t>
+        </is>
+      </c>
+      <c r="G149" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H149" s="12" t="inlineStr">
+        <is>
+          <t>--from *필수 (시작일자 (YYYYMMDD))</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>analysis</t>
+        </is>
+      </c>
+      <c r="C150" s="12" t="inlineStr">
+        <is>
           <t>instant-volume</t>
         </is>
       </c>
-      <c r="D149" s="12" t="inlineStr">
+      <c r="D150" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis instant-volume</t>
         </is>
       </c>
-      <c r="E149" s="12" t="inlineStr">
+      <c r="E150" s="12" t="inlineStr">
         <is>
           <t>거래원순간거래량 조회</t>
         </is>
       </c>
-      <c r="F149" s="13" t="inlineStr">
+      <c r="F150" s="13" t="inlineStr">
         <is>
           <t>ka10052</t>
         </is>
       </c>
-      <c r="G149" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H149" s="12" t="inlineStr">
+      <c r="G150" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H150" s="12" t="inlineStr">
         <is>
           <t>--broker *필수 (회원사코드)
 --code (종목코드 (선택))
@@ -6723,43 +6773,43 @@
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="12" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B150" s="12" t="inlineStr">
+      <c r="B151" s="12" t="inlineStr">
         <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C150" s="12" t="inlineStr">
+      <c r="C151" s="12" t="inlineStr">
         <is>
           <t>open-change</t>
         </is>
       </c>
-      <c r="D150" s="12" t="inlineStr">
+      <c r="D151" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis open-change</t>
         </is>
       </c>
-      <c r="E150" s="12" t="inlineStr">
+      <c r="E151" s="12" t="inlineStr">
         <is>
           <t>시가대비등락률 조회</t>
         </is>
       </c>
-      <c r="F150" s="13" t="inlineStr">
+      <c r="F151" s="13" t="inlineStr">
         <is>
           <t>ka10028</t>
         </is>
       </c>
-      <c r="G150" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H150" s="12" t="inlineStr">
+      <c r="G151" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H151" s="12" t="inlineStr">
         <is>
           <t>--sort [1, 2, 3, 4] 기본:1 (정렬구분 (1=시가, 2=고가, 3=저가, 4=기준가))
 --volume-cond (거래량조건)
@@ -6773,86 +6823,86 @@
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="12" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B151" s="12" t="inlineStr">
+      <c r="B152" s="12" t="inlineStr">
         <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C151" s="12" t="inlineStr">
+      <c r="C152" s="12" t="inlineStr">
         <is>
           <t>per-rank</t>
         </is>
       </c>
-      <c r="D151" s="12" t="inlineStr">
+      <c r="D152" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis per-rank</t>
         </is>
       </c>
-      <c r="E151" s="12" t="inlineStr">
+      <c r="E152" s="12" t="inlineStr">
         <is>
           <t>고저PER 조회</t>
         </is>
       </c>
-      <c r="F151" s="13" t="inlineStr">
+      <c r="F152" s="13" t="inlineStr">
         <is>
           <t>ka10026</t>
         </is>
       </c>
-      <c r="G151" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H151" s="12" t="inlineStr">
+      <c r="G152" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H152" s="12" t="inlineStr">
         <is>
           <t>--type [low-pbr, high-pbr, low-per, high-per, low-roe, high-roe] 기본:low-per (PER구분 (low-pbr/high-pbr/low-per/high-per/low-roe/high-roe))
 --exchange [KRX, NXT, all] 기본:all (거래소구분 (KRX/NXT/all))</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="12" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B152" s="12" t="inlineStr">
+      <c r="B153" s="12" t="inlineStr">
         <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C152" s="12" t="inlineStr">
+      <c r="C153" s="12" t="inlineStr">
         <is>
           <t>price-cluster</t>
         </is>
       </c>
-      <c r="D152" s="12" t="inlineStr">
+      <c r="D153" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis price-cluster</t>
         </is>
       </c>
-      <c r="E152" s="12" t="inlineStr">
+      <c r="E153" s="12" t="inlineStr">
         <is>
           <t>매물대집중 조회</t>
         </is>
       </c>
-      <c r="F152" s="13" t="inlineStr">
+      <c r="F153" s="13" t="inlineStr">
         <is>
           <t>ka10025</t>
         </is>
       </c>
-      <c r="G152" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H152" s="12" t="inlineStr">
+      <c r="G153" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H153" s="12" t="inlineStr">
         <is>
           <t>--market [all, kospi, kosdaq] 기본:all (시장구분 (all/kospi/kosdaq))
 --ratio 기본:50 (매물집중비율 (0~100))
@@ -6863,43 +6913,43 @@
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="12" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B153" s="12" t="inlineStr">
+      <c r="B154" s="12" t="inlineStr">
         <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C153" s="12" t="inlineStr">
+      <c r="C154" s="12" t="inlineStr">
         <is>
           <t>trader-analysis</t>
         </is>
       </c>
-      <c r="D153" s="12" t="inlineStr">
+      <c r="D154" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis trader-analysis</t>
         </is>
       </c>
-      <c r="E153" s="12" t="inlineStr">
+      <c r="E154" s="12" t="inlineStr">
         <is>
           <t>거래원매물대분석 조회</t>
         </is>
       </c>
-      <c r="F153" s="13" t="inlineStr">
+      <c r="F154" s="13" t="inlineStr">
         <is>
           <t>ka10043</t>
         </is>
       </c>
-      <c r="G153" s="12" t="inlineStr">
+      <c r="G154" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H153" s="12" t="inlineStr">
+      <c r="H154" s="12" t="inlineStr">
         <is>
           <t>--from *필수 (시작일자 (YYYYMMDD))
 --to *필수 (종료일자 (YYYYMMDD))
@@ -6912,43 +6962,43 @@
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="12" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B154" s="12" t="inlineStr">
+      <c r="B155" s="12" t="inlineStr">
         <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C154" s="12" t="inlineStr">
+      <c r="C155" s="12" t="inlineStr">
         <is>
           <t>vi-trigger</t>
         </is>
       </c>
-      <c r="D154" s="12" t="inlineStr">
+      <c r="D155" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis vi-trigger</t>
         </is>
       </c>
-      <c r="E154" s="12" t="inlineStr">
+      <c r="E155" s="12" t="inlineStr">
         <is>
           <t>변동성완화장치(VI) 발동종목 조회</t>
         </is>
       </c>
-      <c r="F154" s="13" t="inlineStr">
+      <c r="F155" s="13" t="inlineStr">
         <is>
           <t>ka10054</t>
         </is>
       </c>
-      <c r="G154" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H154" s="12" t="inlineStr">
+      <c r="G155" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H155" s="12" t="inlineStr">
         <is>
           <t>--market [all, kospi, kosdaq] 기본:all (시장구분 (all/kospi/kosdaq))
 --session [0, 1, 2] (장전구분 (0=전체, 1=정규시장, 2=시간외단일가))
@@ -6966,43 +7016,43 @@
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="12" t="inlineStr">
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B155" s="12" t="inlineStr">
+      <c r="B156" s="12" t="inlineStr">
         <is>
           <t>analysis</t>
         </is>
       </c>
-      <c r="C155" s="12" t="inlineStr">
+      <c r="C156" s="12" t="inlineStr">
         <is>
           <t>volume-renewal</t>
         </is>
       </c>
-      <c r="D155" s="12" t="inlineStr">
+      <c r="D156" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock analysis volume-renewal</t>
         </is>
       </c>
-      <c r="E155" s="12" t="inlineStr">
+      <c r="E156" s="12" t="inlineStr">
         <is>
           <t>거래량갱신 조회</t>
         </is>
       </c>
-      <c r="F155" s="13" t="inlineStr">
+      <c r="F156" s="13" t="inlineStr">
         <is>
           <t>ka10024</t>
         </is>
       </c>
-      <c r="G155" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H155" s="12" t="inlineStr">
+      <c r="G156" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H156" s="12" t="inlineStr">
         <is>
           <t>--market [all, kospi, kosdaq] 기본:all (시장구분 (all/kospi/kosdaq))
 --cycle [5, 10, 20, 60, 250] 기본:20 (주기구분 (5/10/20/60/250일))
@@ -7011,48 +7061,6 @@
         </is>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B156" s="12" t="inlineStr">
-        <is>
-          <t>analysis</t>
-        </is>
-      </c>
-      <c r="C156" s="12" t="inlineStr">
-        <is>
-          <t>warrant</t>
-        </is>
-      </c>
-      <c r="D156" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock analysis warrant</t>
-        </is>
-      </c>
-      <c r="E156" s="12" t="inlineStr">
-        <is>
-          <t>신주인수권전체시세 조회</t>
-        </is>
-      </c>
-      <c r="F156" s="13" t="inlineStr">
-        <is>
-          <t>ka10011</t>
-        </is>
-      </c>
-      <c r="G156" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H156" s="12" t="inlineStr">
-        <is>
-          <t>--type [00, 05, 07] 기본:00 (신주인수권구분 (00=전체, 05=신주인수권증권, 07=신주인수권증서))</t>
-        </is>
-      </c>
-    </row>
     <row r="157">
       <c r="A157" s="12" t="inlineStr">
         <is>
@@ -7061,27 +7069,27 @@
       </c>
       <c r="B157" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>analysis</t>
         </is>
       </c>
       <c r="C157" s="12" t="inlineStr">
         <is>
-          <t>brokers</t>
+          <t>warrant</t>
         </is>
       </c>
       <c r="D157" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock brokers</t>
+          <t>kiwoom stock analysis warrant</t>
         </is>
       </c>
       <c r="E157" s="12" t="inlineStr">
         <is>
-          <t>회원사(증권사) 리스트 조회</t>
+          <t>신주인수권전체시세 조회</t>
         </is>
       </c>
       <c r="F157" s="13" t="inlineStr">
         <is>
-          <t>ka10102</t>
+          <t>ka10011</t>
         </is>
       </c>
       <c r="G157" s="12" t="inlineStr">
@@ -7091,7 +7099,7 @@
       </c>
       <c r="H157" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--type [00, 05, 07] 기본:00 (신주인수권구분 (00=전체, 05=신주인수권증권, 07=신주인수권증서))</t>
         </is>
       </c>
     </row>
@@ -7103,31 +7111,73 @@
       </c>
       <c r="B158" s="12" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C158" s="12" t="inlineStr">
+        <is>
+          <t>brokers</t>
+        </is>
+      </c>
+      <c r="D158" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock brokers</t>
+        </is>
+      </c>
+      <c r="E158" s="12" t="inlineStr">
+        <is>
+          <t>회원사(증권사) 리스트 조회</t>
+        </is>
+      </c>
+      <c r="F158" s="13" t="inlineStr">
+        <is>
+          <t>ka10102</t>
+        </is>
+      </c>
+      <c r="G158" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H158" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B159" s="12" t="inlineStr">
+        <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C158" s="12" t="inlineStr">
+      <c r="C159" s="12" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="D158" s="12" t="inlineStr">
+      <c r="D159" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart day</t>
         </is>
       </c>
-      <c r="E158" s="12" t="inlineStr">
+      <c r="E159" s="12" t="inlineStr">
         <is>
           <t>일봉 차트 조회 (국내 ka10081 / 미국 usa06012)</t>
         </is>
       </c>
-      <c r="F158" s="13" t="inlineStr"/>
-      <c r="G158" s="12" t="inlineStr">
+      <c r="F159" s="13" t="inlineStr"/>
+      <c r="G159" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H158" s="12" t="inlineStr">
+      <c r="H159" s="12" t="inlineStr">
         <is>
           <t>--base-date *필수 (기준일자 (YYYYMMDD))
 --adjusted [0, 1] (수정주가구분 (0=미적용, 1=적용))
@@ -7136,43 +7186,43 @@
         </is>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" s="12" t="inlineStr">
+    <row r="160">
+      <c r="A160" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B159" s="12" t="inlineStr">
+      <c r="B160" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C159" s="12" t="inlineStr">
+      <c r="C160" s="12" t="inlineStr">
         <is>
           <t>intraday-investor</t>
         </is>
       </c>
-      <c r="D159" s="12" t="inlineStr">
+      <c r="D160" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart intraday-investor</t>
         </is>
       </c>
-      <c r="E159" s="12" t="inlineStr">
+      <c r="E160" s="12" t="inlineStr">
         <is>
           <t>장중투자자별매매 차트 조회</t>
         </is>
       </c>
-      <c r="F159" s="13" t="inlineStr">
+      <c r="F160" s="13" t="inlineStr">
         <is>
           <t>ka10064</t>
         </is>
       </c>
-      <c r="G159" s="12" t="inlineStr">
+      <c r="G160" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H159" s="12" t="inlineStr">
+      <c r="H160" s="12" t="inlineStr">
         <is>
           <t>--market [kospi, kosdaq] 기본:kospi (시장구분 (kospi/kosdaq))
 --amount-qty [1, 2] 기본:1 (금액수량구분 (1=금액, 2=수량))
@@ -7180,43 +7230,43 @@
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" s="12" t="inlineStr">
+    <row r="161">
+      <c r="A161" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B160" s="12" t="inlineStr">
+      <c r="B161" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C160" s="12" t="inlineStr">
+      <c r="C161" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="D160" s="12" t="inlineStr">
+      <c r="D161" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart investor</t>
         </is>
       </c>
-      <c r="E160" s="12" t="inlineStr">
+      <c r="E161" s="12" t="inlineStr">
         <is>
           <t>종목별투자자기관별 차트 조회</t>
         </is>
       </c>
-      <c r="F160" s="13" t="inlineStr">
+      <c r="F161" s="13" t="inlineStr">
         <is>
           <t>ka10060</t>
         </is>
       </c>
-      <c r="G160" s="12" t="inlineStr">
+      <c r="G161" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H160" s="12" t="inlineStr">
+      <c r="H161" s="12" t="inlineStr">
         <is>
           <t>--date *필수 (일자 (YYYYMMDD))
 --amount-qty [1, 2] 기본:1 (금액수량구분 (1=금액, 2=수량))
@@ -7225,39 +7275,39 @@
         </is>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" s="12" t="inlineStr">
+    <row r="162">
+      <c r="A162" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B161" s="12" t="inlineStr">
+      <c r="B162" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C161" s="12" t="inlineStr">
+      <c r="C162" s="12" t="inlineStr">
         <is>
           <t>minute</t>
         </is>
       </c>
-      <c r="D161" s="12" t="inlineStr">
+      <c r="D162" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart minute</t>
         </is>
       </c>
-      <c r="E161" s="12" t="inlineStr">
+      <c r="E162" s="12" t="inlineStr">
         <is>
           <t>분봉 차트 조회 (국내 ka10080 / 미국 usa06011)</t>
         </is>
       </c>
-      <c r="F161" s="13" t="inlineStr"/>
-      <c r="G161" s="12" t="inlineStr">
+      <c r="F162" s="13" t="inlineStr"/>
+      <c r="G162" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H161" s="12" t="inlineStr">
+      <c r="H162" s="12" t="inlineStr">
         <is>
           <t>--interval [1, 3, 5, 10, 15, 30, 45, 60] 기본:5 (분봉 간격 (1/3/5/10/15/30/45/60))
 --adjusted [0, 1] (수정주가구분 (0=미적용, 1=적용))
@@ -7267,39 +7317,39 @@
         </is>
       </c>
     </row>
-    <row r="162">
-      <c r="A162" s="12" t="inlineStr">
+    <row r="163">
+      <c r="A163" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B162" s="12" t="inlineStr">
+      <c r="B163" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C162" s="12" t="inlineStr">
+      <c r="C163" s="12" t="inlineStr">
         <is>
           <t>month</t>
         </is>
       </c>
-      <c r="D162" s="12" t="inlineStr">
+      <c r="D163" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart month</t>
         </is>
       </c>
-      <c r="E162" s="12" t="inlineStr">
+      <c r="E163" s="12" t="inlineStr">
         <is>
           <t>월봉 차트 조회 (국내 ka10083 / 미국 usa06014)</t>
         </is>
       </c>
-      <c r="F162" s="13" t="inlineStr"/>
-      <c r="G162" s="12" t="inlineStr">
+      <c r="F163" s="13" t="inlineStr"/>
+      <c r="G163" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H162" s="12" t="inlineStr">
+      <c r="H163" s="12" t="inlineStr">
         <is>
           <t>--base-date *필수 (기준일자 (YYYYMMDD))
 --adjusted [0, 1] (수정주가구분 (0=미적용, 1=적용))
@@ -7308,39 +7358,39 @@
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="A163" s="12" t="inlineStr">
+    <row r="164">
+      <c r="A164" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B163" s="12" t="inlineStr">
+      <c r="B164" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C163" s="12" t="inlineStr">
+      <c r="C164" s="12" t="inlineStr">
         <is>
           <t>tick</t>
         </is>
       </c>
-      <c r="D163" s="12" t="inlineStr">
+      <c r="D164" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart tick</t>
         </is>
       </c>
-      <c r="E163" s="12" t="inlineStr">
+      <c r="E164" s="12" t="inlineStr">
         <is>
           <t>틱 차트 조회 (국내 ka10079 / 미국 usa06010)</t>
         </is>
       </c>
-      <c r="F163" s="13" t="inlineStr"/>
-      <c r="G163" s="12" t="inlineStr">
+      <c r="F164" s="13" t="inlineStr"/>
+      <c r="G164" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H163" s="12" t="inlineStr">
+      <c r="H164" s="12" t="inlineStr">
         <is>
           <t>--range [1, 3, 5, 10, 30] 기본:1 (틱범위 (1/3/5/10/30))
 --adjusted [0, 1] (수정주가구분 (0=미적용, 1=적용))
@@ -7349,39 +7399,39 @@
         </is>
       </c>
     </row>
-    <row r="164">
-      <c r="A164" s="12" t="inlineStr">
+    <row r="165">
+      <c r="A165" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B164" s="12" t="inlineStr">
+      <c r="B165" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C164" s="12" t="inlineStr">
+      <c r="C165" s="12" t="inlineStr">
         <is>
           <t>week</t>
         </is>
       </c>
-      <c r="D164" s="12" t="inlineStr">
+      <c r="D165" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart week</t>
         </is>
       </c>
-      <c r="E164" s="12" t="inlineStr">
+      <c r="E165" s="12" t="inlineStr">
         <is>
           <t>주봉 차트 조회 (국내 ka10082 / 미국 usa06013)</t>
         </is>
       </c>
-      <c r="F164" s="13" t="inlineStr"/>
-      <c r="G164" s="12" t="inlineStr">
+      <c r="F165" s="13" t="inlineStr"/>
+      <c r="G165" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H164" s="12" t="inlineStr">
+      <c r="H165" s="12" t="inlineStr">
         <is>
           <t>--base-date *필수 (기준일자 (YYYYMMDD))
 --adjusted [0, 1] (수정주가구분 (0=미적용, 1=적용))
@@ -7390,39 +7440,39 @@
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="A165" s="12" t="inlineStr">
+    <row r="166">
+      <c r="A166" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B165" s="12" t="inlineStr">
+      <c r="B166" s="12" t="inlineStr">
         <is>
           <t>chart</t>
         </is>
       </c>
-      <c r="C165" s="12" t="inlineStr">
+      <c r="C166" s="12" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="D165" s="12" t="inlineStr">
+      <c r="D166" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock chart year</t>
         </is>
       </c>
-      <c r="E165" s="12" t="inlineStr">
+      <c r="E166" s="12" t="inlineStr">
         <is>
           <t>년봉 차트 조회 (국내 ka10094 / 미국 usa06015)</t>
         </is>
       </c>
-      <c r="F165" s="13" t="inlineStr"/>
-      <c r="G165" s="12" t="inlineStr">
+      <c r="F166" s="13" t="inlineStr"/>
+      <c r="G166" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H165" s="12" t="inlineStr">
+      <c r="H166" s="12" t="inlineStr">
         <is>
           <t>--base-date *필수 (기준일자 (YYYYMMDD))
 --adjusted [0, 1] (수정주가구분 (0=미적용, 1=적용))
@@ -7431,48 +7481,6 @@
         </is>
       </c>
     </row>
-    <row r="166">
-      <c r="A166" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B166" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C166" s="12" t="inlineStr">
-        <is>
-          <t>compare</t>
-        </is>
-      </c>
-      <c r="D166" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock compare</t>
-        </is>
-      </c>
-      <c r="E166" s="12" t="inlineStr">
-        <is>
-          <t>종목 비교 (2개 이상)</t>
-        </is>
-      </c>
-      <c r="F166" s="13" t="inlineStr">
-        <is>
-          <t>ka10001</t>
-        </is>
-      </c>
-      <c r="G166" s="12" t="inlineStr">
-        <is>
-          <t>CODES (복수) (필수)</t>
-        </is>
-      </c>
-      <c r="H166" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
     <row r="167">
       <c r="A167" s="12" t="inlineStr">
         <is>
@@ -7481,32 +7489,32 @@
       </c>
       <c r="B167" s="12" t="inlineStr">
         <is>
-          <t>credit</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C167" s="12" t="inlineStr">
         <is>
-          <t>available</t>
+          <t>compare</t>
         </is>
       </c>
       <c r="D167" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock credit available</t>
+          <t>kiwoom stock compare</t>
         </is>
       </c>
       <c r="E167" s="12" t="inlineStr">
         <is>
-          <t>신용융자 가능종목 조회</t>
+          <t>종목 비교 (2개 이상)</t>
         </is>
       </c>
       <c r="F167" s="13" t="inlineStr">
         <is>
-          <t>kt20016</t>
+          <t>ka10001</t>
         </is>
       </c>
       <c r="G167" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H167" s="12" t="inlineStr">
@@ -7528,22 +7536,22 @@
       </c>
       <c r="C168" s="12" t="inlineStr">
         <is>
-          <t>inquiry</t>
+          <t>available</t>
         </is>
       </c>
       <c r="D168" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock credit inquiry</t>
+          <t>kiwoom stock credit available</t>
         </is>
       </c>
       <c r="E168" s="12" t="inlineStr">
         <is>
-          <t>신용융자 가능문의</t>
+          <t>신용융자 가능종목 조회</t>
         </is>
       </c>
       <c r="F168" s="13" t="inlineStr">
         <is>
-          <t>kt20017</t>
+          <t>kt20016</t>
         </is>
       </c>
       <c r="G168" s="12" t="inlineStr">
@@ -7570,78 +7578,78 @@
       </c>
       <c r="C169" s="12" t="inlineStr">
         <is>
+          <t>inquiry</t>
+        </is>
+      </c>
+      <c r="D169" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock credit inquiry</t>
+        </is>
+      </c>
+      <c r="E169" s="12" t="inlineStr">
+        <is>
+          <t>신용융자 가능문의</t>
+        </is>
+      </c>
+      <c r="F169" s="13" t="inlineStr">
+        <is>
+          <t>kt20017</t>
+        </is>
+      </c>
+      <c r="G169" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H169" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B170" s="12" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+      <c r="C170" s="12" t="inlineStr">
+        <is>
           <t>trend</t>
         </is>
       </c>
-      <c r="D169" s="12" t="inlineStr">
+      <c r="D170" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock credit trend</t>
         </is>
       </c>
-      <c r="E169" s="12" t="inlineStr">
+      <c r="E170" s="12" t="inlineStr">
         <is>
           <t>신용매매동향 조회</t>
         </is>
       </c>
-      <c r="F169" s="13" t="inlineStr">
+      <c r="F170" s="13" t="inlineStr">
         <is>
           <t>ka10013</t>
         </is>
       </c>
-      <c r="G169" s="12" t="inlineStr">
+      <c r="G170" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H169" s="12" t="inlineStr">
+      <c r="H170" s="12" t="inlineStr">
         <is>
           <t>--date *필수 (일자 (YYYYMMDD))
 --type [loan, short-sell] 기본:loan (구분 (loan=융자, short-sell=대주))</t>
         </is>
       </c>
     </row>
-    <row r="170">
-      <c r="A170" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B170" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C170" s="12" t="inlineStr">
-        <is>
-          <t>daily</t>
-        </is>
-      </c>
-      <c r="D170" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock daily</t>
-        </is>
-      </c>
-      <c r="E170" s="12" t="inlineStr">
-        <is>
-          <t>일/주/월별 시세 조회</t>
-        </is>
-      </c>
-      <c r="F170" s="13" t="inlineStr">
-        <is>
-          <t>ka10005</t>
-        </is>
-      </c>
-      <c r="G170" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H170" s="12" t="inlineStr">
-        <is>
-          <t>--type [day, week, month] 기본:day (조회 구분 (day/week/month))</t>
-        </is>
-      </c>
-    </row>
     <row r="171">
       <c r="A171" s="12" t="inlineStr">
         <is>
@@ -7655,78 +7663,78 @@
       </c>
       <c r="C171" s="12" t="inlineStr">
         <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="D171" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock daily</t>
+        </is>
+      </c>
+      <c r="E171" s="12" t="inlineStr">
+        <is>
+          <t>일/주/월별 시세 조회</t>
+        </is>
+      </c>
+      <c r="F171" s="13" t="inlineStr">
+        <is>
+          <t>ka10005</t>
+        </is>
+      </c>
+      <c r="G171" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H171" s="12" t="inlineStr">
+        <is>
+          <t>--type [day, week, month] 기본:day (조회 구분 (day/week/month))</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B172" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C172" s="12" t="inlineStr">
+        <is>
           <t>daily-price</t>
         </is>
       </c>
-      <c r="D171" s="12" t="inlineStr">
+      <c r="D172" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock daily-price</t>
         </is>
       </c>
-      <c r="E171" s="12" t="inlineStr">
+      <c r="E172" s="12" t="inlineStr">
         <is>
           <t>일별주가 조회</t>
         </is>
       </c>
-      <c r="F171" s="13" t="inlineStr">
+      <c r="F172" s="13" t="inlineStr">
         <is>
           <t>ka10086</t>
         </is>
       </c>
-      <c r="G171" s="12" t="inlineStr">
+      <c r="G172" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H171" s="12" t="inlineStr">
+      <c r="H172" s="12" t="inlineStr">
         <is>
           <t>--date *필수 (조회일자 (YYYYMMDD))
 --display [0, 1] (표시구분 (0=수량, 1=금액백만원))</t>
         </is>
       </c>
     </row>
-    <row r="172">
-      <c r="A172" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B172" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C172" s="12" t="inlineStr">
-        <is>
-          <t>daily-strength</t>
-        </is>
-      </c>
-      <c r="D172" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock daily-strength</t>
-        </is>
-      </c>
-      <c r="E172" s="12" t="inlineStr">
-        <is>
-          <t>체결강도추이 일별</t>
-        </is>
-      </c>
-      <c r="F172" s="13" t="inlineStr">
-        <is>
-          <t>ka10047</t>
-        </is>
-      </c>
-      <c r="G172" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H172" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
     <row r="173">
       <c r="A173" s="12" t="inlineStr">
         <is>
@@ -7740,22 +7748,22 @@
       </c>
       <c r="C173" s="12" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>daily-strength</t>
         </is>
       </c>
       <c r="D173" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock detail</t>
+          <t>kiwoom stock daily-strength</t>
         </is>
       </c>
       <c r="E173" s="12" t="inlineStr">
         <is>
-          <t>종목정보 상세 조회</t>
+          <t>체결강도추이 일별</t>
         </is>
       </c>
       <c r="F173" s="13" t="inlineStr">
         <is>
-          <t>ka10100</t>
+          <t>ka10047</t>
         </is>
       </c>
       <c r="G173" s="12" t="inlineStr">
@@ -7782,22 +7790,22 @@
       </c>
       <c r="C174" s="12" t="inlineStr">
         <is>
-          <t>exec</t>
+          <t>detail</t>
         </is>
       </c>
       <c r="D174" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock exec</t>
+          <t>kiwoom stock detail</t>
         </is>
       </c>
       <c r="E174" s="12" t="inlineStr">
         <is>
-          <t>체결정보 조회</t>
+          <t>종목정보 상세 조회</t>
         </is>
       </c>
       <c r="F174" s="13" t="inlineStr">
         <is>
-          <t>ka10003</t>
+          <t>ka10100</t>
         </is>
       </c>
       <c r="G174" s="12" t="inlineStr">
@@ -7824,22 +7832,22 @@
       </c>
       <c r="C175" s="12" t="inlineStr">
         <is>
-          <t>foreign</t>
+          <t>exec</t>
         </is>
       </c>
       <c r="D175" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock foreign</t>
+          <t>kiwoom stock exec</t>
         </is>
       </c>
       <c r="E175" s="12" t="inlineStr">
         <is>
-          <t>외국인 종목별 매매동향 조회</t>
+          <t>체결정보 조회</t>
         </is>
       </c>
       <c r="F175" s="13" t="inlineStr">
         <is>
-          <t>ka10008</t>
+          <t>ka10003</t>
         </is>
       </c>
       <c r="G175" s="12" t="inlineStr">
@@ -7866,20 +7874,24 @@
       </c>
       <c r="C176" s="12" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>foreign</t>
         </is>
       </c>
       <c r="D176" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock info</t>
+          <t>kiwoom stock foreign</t>
         </is>
       </c>
       <c r="E176" s="12" t="inlineStr">
         <is>
-          <t>종목 기본정보 조회</t>
-        </is>
-      </c>
-      <c r="F176" s="13" t="inlineStr"/>
+          <t>외국인 종목별 매매동향 조회</t>
+        </is>
+      </c>
+      <c r="F176" s="13" t="inlineStr">
+        <is>
+          <t>ka10008</t>
+        </is>
+      </c>
       <c r="G176" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -7887,7 +7899,7 @@
       </c>
       <c r="H176" s="12" t="inlineStr">
         <is>
-          <t>--exchange [nasdaq, nyse, amex] (미국 거래소 (미국 종목 강제 라우팅))</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -7904,24 +7916,20 @@
       </c>
       <c r="C177" s="12" t="inlineStr">
         <is>
-          <t>institution</t>
+          <t>info</t>
         </is>
       </c>
       <c r="D177" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock institution</t>
+          <t>kiwoom stock info</t>
         </is>
       </c>
       <c r="E177" s="12" t="inlineStr">
         <is>
-          <t>주식기관 조회</t>
-        </is>
-      </c>
-      <c r="F177" s="13" t="inlineStr">
-        <is>
-          <t>ka10009</t>
-        </is>
-      </c>
+          <t>종목 기본정보 조회</t>
+        </is>
+      </c>
+      <c r="F177" s="13" t="inlineStr"/>
       <c r="G177" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -7929,7 +7937,7 @@
       </c>
       <c r="H177" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--exchange [nasdaq, nyse, amex] (미국 거래소 (미국 종목 강제 라우팅))</t>
         </is>
       </c>
     </row>
@@ -7941,35 +7949,77 @@
       </c>
       <c r="B178" s="12" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C178" s="12" t="inlineStr">
+        <is>
+          <t>institution</t>
+        </is>
+      </c>
+      <c r="D178" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock institution</t>
+        </is>
+      </c>
+      <c r="E178" s="12" t="inlineStr">
+        <is>
+          <t>주식기관 조회</t>
+        </is>
+      </c>
+      <c r="F178" s="13" t="inlineStr">
+        <is>
+          <t>ka10009</t>
+        </is>
+      </c>
+      <c r="G178" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H178" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B179" s="12" t="inlineStr">
+        <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C178" s="12" t="inlineStr">
+      <c r="C179" s="12" t="inlineStr">
         <is>
           <t>after-close</t>
         </is>
       </c>
-      <c r="D178" s="12" t="inlineStr">
+      <c r="D179" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor after-close</t>
         </is>
       </c>
-      <c r="E178" s="12" t="inlineStr">
+      <c r="E179" s="12" t="inlineStr">
         <is>
           <t>장마감후투자자별매매 조회</t>
         </is>
       </c>
-      <c r="F178" s="13" t="inlineStr">
+      <c r="F179" s="13" t="inlineStr">
         <is>
           <t>ka10066</t>
         </is>
       </c>
-      <c r="G178" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H178" s="12" t="inlineStr">
+      <c r="G179" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H179" s="12" t="inlineStr">
         <is>
           <t>--market [kospi, kosdaq] 기본:kospi (시장구분 (kospi/kosdaq))
 --amount-qty [1, 2] 기본:1 (금액수량구분 (1=금액, 2=수량))
@@ -7978,43 +8028,43 @@
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="A179" s="12" t="inlineStr">
+    <row r="180">
+      <c r="A180" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B179" s="12" t="inlineStr">
+      <c r="B180" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C179" s="12" t="inlineStr">
+      <c r="C180" s="12" t="inlineStr">
         <is>
           <t>by-stock</t>
         </is>
       </c>
-      <c r="D179" s="12" t="inlineStr">
+      <c r="D180" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor by-stock</t>
         </is>
       </c>
-      <c r="E179" s="12" t="inlineStr">
+      <c r="E180" s="12" t="inlineStr">
         <is>
           <t>종목별투자자기관별 조회</t>
         </is>
       </c>
-      <c r="F179" s="13" t="inlineStr">
+      <c r="F180" s="13" t="inlineStr">
         <is>
           <t>ka10059</t>
         </is>
       </c>
-      <c r="G179" s="12" t="inlineStr">
+      <c r="G180" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H179" s="12" t="inlineStr">
+      <c r="H180" s="12" t="inlineStr">
         <is>
           <t>--date *필수 (일자 (YYYYMMDD))
 --amount-qty [1, 2] 기본:1 (금액수량구분 (1=금액, 2=수량))
@@ -8023,43 +8073,43 @@
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="A180" s="12" t="inlineStr">
+    <row r="181">
+      <c r="A181" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B180" s="12" t="inlineStr">
+      <c r="B181" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C180" s="12" t="inlineStr">
+      <c r="C181" s="12" t="inlineStr">
         <is>
           <t>by-stock-total</t>
         </is>
       </c>
-      <c r="D180" s="12" t="inlineStr">
+      <c r="D181" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor by-stock-total</t>
         </is>
       </c>
-      <c r="E180" s="12" t="inlineStr">
+      <c r="E181" s="12" t="inlineStr">
         <is>
           <t>종목별투자자기관별합계 조회</t>
         </is>
       </c>
-      <c r="F180" s="13" t="inlineStr">
+      <c r="F181" s="13" t="inlineStr">
         <is>
           <t>ka10061</t>
         </is>
       </c>
-      <c r="G180" s="12" t="inlineStr">
+      <c r="G181" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H180" s="12" t="inlineStr">
+      <c r="H181" s="12" t="inlineStr">
         <is>
           <t>--from *필수 (시작일자 (YYYYMMDD))
 --to *필수 (종료일자 (YYYYMMDD))
@@ -8069,43 +8119,43 @@
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="A181" s="12" t="inlineStr">
+    <row r="182">
+      <c r="A182" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B181" s="12" t="inlineStr">
+      <c r="B182" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C181" s="12" t="inlineStr">
+      <c r="C182" s="12" t="inlineStr">
         <is>
           <t>consecutive</t>
         </is>
       </c>
-      <c r="D181" s="12" t="inlineStr">
+      <c r="D182" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor consecutive</t>
         </is>
       </c>
-      <c r="E181" s="12" t="inlineStr">
+      <c r="E182" s="12" t="inlineStr">
         <is>
           <t>기관/외국인 연속매매현황 조회</t>
         </is>
       </c>
-      <c r="F181" s="13" t="inlineStr">
+      <c r="F182" s="13" t="inlineStr">
         <is>
           <t>ka10131</t>
         </is>
       </c>
-      <c r="G181" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H181" s="12" t="inlineStr">
+      <c r="G182" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H182" s="12" t="inlineStr">
         <is>
           <t>--period 기본:5 (기간 (일수))
 --from (시작일자 (YYYYMMDD, 선택))
@@ -8118,43 +8168,43 @@
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="A182" s="12" t="inlineStr">
+    <row r="183">
+      <c r="A183" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B182" s="12" t="inlineStr">
+      <c r="B183" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C182" s="12" t="inlineStr">
+      <c r="C183" s="12" t="inlineStr">
         <is>
           <t>daily-by-investor</t>
         </is>
       </c>
-      <c r="D182" s="12" t="inlineStr">
+      <c r="D183" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor daily-by-investor</t>
         </is>
       </c>
-      <c r="E182" s="12" t="inlineStr">
+      <c r="E183" s="12" t="inlineStr">
         <is>
           <t>투자자별일별매매종목 조회</t>
         </is>
       </c>
-      <c r="F182" s="13" t="inlineStr">
+      <c r="F183" s="13" t="inlineStr">
         <is>
           <t>ka10058</t>
         </is>
       </c>
-      <c r="G182" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H182" s="12" t="inlineStr">
+      <c r="G183" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H183" s="12" t="inlineStr">
         <is>
           <t>--from *필수 (시작일자 (YYYYMMDD))
 --to *필수 (종료일자 (YYYYMMDD))
@@ -8165,43 +8215,43 @@
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="12" t="inlineStr">
+    <row r="184">
+      <c r="A184" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B183" s="12" t="inlineStr">
+      <c r="B184" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C183" s="12" t="inlineStr">
+      <c r="C184" s="12" t="inlineStr">
         <is>
           <t>daily-trade</t>
         </is>
       </c>
-      <c r="D183" s="12" t="inlineStr">
+      <c r="D184" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor daily-trade</t>
         </is>
       </c>
-      <c r="E183" s="12" t="inlineStr">
+      <c r="E184" s="12" t="inlineStr">
         <is>
           <t>일별기관매매종목 조회</t>
         </is>
       </c>
-      <c r="F183" s="13" t="inlineStr">
+      <c r="F184" s="13" t="inlineStr">
         <is>
           <t>ka10044</t>
         </is>
       </c>
-      <c r="G183" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H183" s="12" t="inlineStr">
+      <c r="G184" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H184" s="12" t="inlineStr">
         <is>
           <t>--from *필수 (시작일자 (YYYYMMDD))
 --to *필수 (종료일자 (YYYYMMDD))
@@ -8211,43 +8261,43 @@
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="A184" s="12" t="inlineStr">
+    <row r="185">
+      <c r="A185" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B184" s="12" t="inlineStr">
+      <c r="B185" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C184" s="12" t="inlineStr">
+      <c r="C185" s="12" t="inlineStr">
         <is>
           <t>intraday</t>
         </is>
       </c>
-      <c r="D184" s="12" t="inlineStr">
+      <c r="D185" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor intraday</t>
         </is>
       </c>
-      <c r="E184" s="12" t="inlineStr">
+      <c r="E185" s="12" t="inlineStr">
         <is>
           <t>장중투자자별매매 조회</t>
         </is>
       </c>
-      <c r="F184" s="13" t="inlineStr">
+      <c r="F185" s="13" t="inlineStr">
         <is>
           <t>ka10063</t>
         </is>
       </c>
-      <c r="G184" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H184" s="12" t="inlineStr">
+      <c r="G185" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H185" s="12" t="inlineStr">
         <is>
           <t>--market [kospi, kosdaq] 기본:kospi (시장구분 (kospi/kosdaq))
 --amount-qty 기본:1 (금액수량구분 (1=금액&amp;수량))
@@ -8258,43 +8308,43 @@
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" s="12" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B185" s="12" t="inlineStr">
+      <c r="B186" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C185" s="12" t="inlineStr">
+      <c r="C186" s="12" t="inlineStr">
         <is>
           <t>program-by-stock</t>
         </is>
       </c>
-      <c r="D185" s="12" t="inlineStr">
+      <c r="D186" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor program-by-stock</t>
         </is>
       </c>
-      <c r="E185" s="12" t="inlineStr">
+      <c r="E186" s="12" t="inlineStr">
         <is>
           <t>종목별프로그램매매현황 조회</t>
         </is>
       </c>
-      <c r="F185" s="13" t="inlineStr">
+      <c r="F186" s="13" t="inlineStr">
         <is>
           <t>ka90004</t>
         </is>
       </c>
-      <c r="G185" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H185" s="12" t="inlineStr">
+      <c r="G186" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H186" s="12" t="inlineStr">
         <is>
           <t>--date *필수 (일자 (YYYYMMDD))
 --market [kospi, kosdaq] 기본:kospi (시장구분 (kospi/kosdaq))
@@ -8302,43 +8352,43 @@
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="A186" s="12" t="inlineStr">
+    <row r="187">
+      <c r="A187" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B186" s="12" t="inlineStr">
+      <c r="B187" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C186" s="12" t="inlineStr">
+      <c r="C187" s="12" t="inlineStr">
         <is>
           <t>program-top</t>
         </is>
       </c>
-      <c r="D186" s="12" t="inlineStr">
+      <c r="D187" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor program-top</t>
         </is>
       </c>
-      <c r="E186" s="12" t="inlineStr">
+      <c r="E187" s="12" t="inlineStr">
         <is>
           <t>프로그램순매수상위50 조회</t>
         </is>
       </c>
-      <c r="F186" s="13" t="inlineStr">
+      <c r="F187" s="13" t="inlineStr">
         <is>
           <t>ka90003</t>
         </is>
       </c>
-      <c r="G186" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H186" s="12" t="inlineStr">
+      <c r="G187" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H187" s="12" t="inlineStr">
         <is>
           <t>--trade [1, 2] 기본:2 (매매구분 (1=순매도, 2=순매수))
 --amount-qty [1, 2] 기본:1 (금액수량구분 (1=금액, 2=수량))
@@ -8347,43 +8397,43 @@
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="12" t="inlineStr">
+    <row r="188">
+      <c r="A188" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B187" s="12" t="inlineStr">
+      <c r="B188" s="12" t="inlineStr">
         <is>
           <t>investor</t>
         </is>
       </c>
-      <c r="C187" s="12" t="inlineStr">
+      <c r="C188" s="12" t="inlineStr">
         <is>
           <t>stock-institution</t>
         </is>
       </c>
-      <c r="D187" s="12" t="inlineStr">
+      <c r="D188" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock investor stock-institution</t>
         </is>
       </c>
-      <c r="E187" s="12" t="inlineStr">
+      <c r="E188" s="12" t="inlineStr">
         <is>
           <t>종목별기관매매추이 조회</t>
         </is>
       </c>
-      <c r="F187" s="13" t="inlineStr">
+      <c r="F188" s="13" t="inlineStr">
         <is>
           <t>ka10045</t>
         </is>
       </c>
-      <c r="G187" s="12" t="inlineStr">
+      <c r="G188" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H187" s="12" t="inlineStr">
+      <c r="H188" s="12" t="inlineStr">
         <is>
           <t>--from *필수 (시작일자 (YYYYMMDD))
 --to *필수 (종료일자 (YYYYMMDD))
@@ -8392,43 +8442,43 @@
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="12" t="inlineStr">
+    <row r="189">
+      <c r="A189" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B188" s="12" t="inlineStr">
+      <c r="B189" s="12" t="inlineStr">
         <is>
           <t>lending</t>
         </is>
       </c>
-      <c r="C188" s="12" t="inlineStr">
+      <c r="C189" s="12" t="inlineStr">
         <is>
           <t>by-stock</t>
         </is>
       </c>
-      <c r="D188" s="12" t="inlineStr">
+      <c r="D189" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock lending by-stock</t>
         </is>
       </c>
-      <c r="E188" s="12" t="inlineStr">
+      <c r="E189" s="12" t="inlineStr">
         <is>
           <t>대차거래추이 종목별 조회</t>
         </is>
       </c>
-      <c r="F188" s="13" t="inlineStr">
+      <c r="F189" s="13" t="inlineStr">
         <is>
           <t>ka20068</t>
         </is>
       </c>
-      <c r="G188" s="12" t="inlineStr">
+      <c r="G189" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H188" s="12" t="inlineStr">
+      <c r="H189" s="12" t="inlineStr">
         <is>
           <t>--from (시작일자 (YYYYMMDD, 선택))
 --to (종료일자 (YYYYMMDD, 선택))
@@ -8436,86 +8486,86 @@
         </is>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="12" t="inlineStr">
+    <row r="190">
+      <c r="A190" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B189" s="12" t="inlineStr">
+      <c r="B190" s="12" t="inlineStr">
         <is>
           <t>lending</t>
         </is>
       </c>
-      <c r="C189" s="12" t="inlineStr">
+      <c r="C190" s="12" t="inlineStr">
         <is>
           <t>detail</t>
         </is>
       </c>
-      <c r="D189" s="12" t="inlineStr">
+      <c r="D190" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock lending detail</t>
         </is>
       </c>
-      <c r="E189" s="12" t="inlineStr">
+      <c r="E190" s="12" t="inlineStr">
         <is>
           <t>대차거래내역 조회</t>
         </is>
       </c>
-      <c r="F189" s="13" t="inlineStr">
+      <c r="F190" s="13" t="inlineStr">
         <is>
           <t>ka90012</t>
         </is>
       </c>
-      <c r="G189" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H189" s="12" t="inlineStr">
+      <c r="G190" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H190" s="12" t="inlineStr">
         <is>
           <t>--date *필수 (일자 (YYYYMMDD))
 --market [kospi, kosdaq] 기본:kospi (시장구분 (kospi/kosdaq))</t>
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="12" t="inlineStr">
+    <row r="191">
+      <c r="A191" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B190" s="12" t="inlineStr">
+      <c r="B191" s="12" t="inlineStr">
         <is>
           <t>lending</t>
         </is>
       </c>
-      <c r="C190" s="12" t="inlineStr">
+      <c r="C191" s="12" t="inlineStr">
         <is>
           <t>top10</t>
         </is>
       </c>
-      <c r="D190" s="12" t="inlineStr">
+      <c r="D191" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock lending top10</t>
         </is>
       </c>
-      <c r="E190" s="12" t="inlineStr">
+      <c r="E191" s="12" t="inlineStr">
         <is>
           <t>대차거래상위10종목 조회</t>
         </is>
       </c>
-      <c r="F190" s="13" t="inlineStr">
+      <c r="F191" s="13" t="inlineStr">
         <is>
           <t>ka10069</t>
         </is>
       </c>
-      <c r="G190" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H190" s="12" t="inlineStr">
+      <c r="G191" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H191" s="12" t="inlineStr">
         <is>
           <t>--from *필수 (시작일자 (YYYYMMDD))
 --to (종료일자 (YYYYMMDD, 선택))
@@ -8523,43 +8573,43 @@
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="12" t="inlineStr">
+    <row r="192">
+      <c r="A192" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B191" s="12" t="inlineStr">
+      <c r="B192" s="12" t="inlineStr">
         <is>
           <t>lending</t>
         </is>
       </c>
-      <c r="C191" s="12" t="inlineStr">
+      <c r="C192" s="12" t="inlineStr">
         <is>
           <t>trend</t>
         </is>
       </c>
-      <c r="D191" s="12" t="inlineStr">
+      <c r="D192" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock lending trend</t>
         </is>
       </c>
-      <c r="E191" s="12" t="inlineStr">
+      <c r="E192" s="12" t="inlineStr">
         <is>
           <t>대차거래추이 조회</t>
         </is>
       </c>
-      <c r="F191" s="13" t="inlineStr">
+      <c r="F192" s="13" t="inlineStr">
         <is>
           <t>ka10068</t>
         </is>
       </c>
-      <c r="G191" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H191" s="12" t="inlineStr">
+      <c r="G192" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H192" s="12" t="inlineStr">
         <is>
           <t>--from (시작일자 (YYYYMMDD, 선택))
 --to (종료일자 (YYYYMMDD, 선택))
@@ -8567,44 +8617,6 @@
         </is>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B192" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C192" s="12" t="inlineStr">
-        <is>
-          <t>orderbook</t>
-        </is>
-      </c>
-      <c r="D192" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock orderbook</t>
-        </is>
-      </c>
-      <c r="E192" s="12" t="inlineStr">
-        <is>
-          <t>호가창 조회</t>
-        </is>
-      </c>
-      <c r="F192" s="13" t="inlineStr"/>
-      <c r="G192" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H192" s="12" t="inlineStr">
-        <is>
-          <t>--exchange [nasdaq, nyse, amex] (미국 거래소 (미국 종목 강제 라우팅))</t>
-        </is>
-      </c>
-    </row>
     <row r="193">
       <c r="A193" s="12" t="inlineStr">
         <is>
@@ -8618,17 +8630,17 @@
       </c>
       <c r="C193" s="12" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>orderbook</t>
         </is>
       </c>
       <c r="D193" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock price</t>
+          <t>kiwoom stock orderbook</t>
         </is>
       </c>
       <c r="E193" s="12" t="inlineStr">
         <is>
-          <t>종목 현재가 간단 조회</t>
+          <t>호가창 조회</t>
         </is>
       </c>
       <c r="F193" s="13" t="inlineStr"/>
@@ -8656,24 +8668,20 @@
       </c>
       <c r="C194" s="12" t="inlineStr">
         <is>
-          <t>quote-info</t>
+          <t>price</t>
         </is>
       </c>
       <c r="D194" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock quote-info</t>
+          <t>kiwoom stock price</t>
         </is>
       </c>
       <c r="E194" s="12" t="inlineStr">
         <is>
-          <t>시세표성정보 조회</t>
-        </is>
-      </c>
-      <c r="F194" s="13" t="inlineStr">
-        <is>
-          <t>ka10007</t>
-        </is>
-      </c>
+          <t>종목 현재가 간단 조회</t>
+        </is>
+      </c>
+      <c r="F194" s="13" t="inlineStr"/>
       <c r="G194" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -8681,7 +8689,7 @@
       </c>
       <c r="H194" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--exchange [nasdaq, nyse, amex] (미국 거래소 (미국 종목 강제 라우팅))</t>
         </is>
       </c>
     </row>
@@ -8698,117 +8706,117 @@
       </c>
       <c r="C195" s="12" t="inlineStr">
         <is>
+          <t>quote-info</t>
+        </is>
+      </c>
+      <c r="D195" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock quote-info</t>
+        </is>
+      </c>
+      <c r="E195" s="12" t="inlineStr">
+        <is>
+          <t>시세표성정보 조회</t>
+        </is>
+      </c>
+      <c r="F195" s="13" t="inlineStr">
+        <is>
+          <t>ka10007</t>
+        </is>
+      </c>
+      <c r="G195" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H195" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B196" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C196" s="12" t="inlineStr">
+        <is>
           <t>search</t>
         </is>
       </c>
-      <c r="D195" s="12" t="inlineStr">
+      <c r="D196" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock search</t>
         </is>
       </c>
-      <c r="E195" s="12" t="inlineStr">
+      <c r="E196" s="12" t="inlineStr">
         <is>
           <t>캐시에서 종목 검색</t>
         </is>
       </c>
-      <c r="F195" s="13" t="inlineStr"/>
-      <c r="G195" s="12" t="inlineStr">
+      <c r="F196" s="13" t="inlineStr"/>
+      <c r="G196" s="12" t="inlineStr">
         <is>
           <t>KEYWORD (선택)</t>
         </is>
       </c>
-      <c r="H195" s="12" t="inlineStr">
+      <c r="H196" s="12" t="inlineStr">
         <is>
           <t>--market [all, kospi, kosdaq, etf, elw, etn, us] 기본:all (시장/유형 필터 (all/kospi/kosdaq/etf/elw/etn/us))
 --exchange [nasdaq, nyse, amex, all] 기본:all (미국 거래소 필터 (--market us 일 때만 사용))</t>
         </is>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="12" t="inlineStr">
+    <row r="197">
+      <c r="A197" s="12" t="inlineStr">
         <is>
           <t>stock</t>
         </is>
       </c>
-      <c r="B196" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C196" s="12" t="inlineStr">
+      <c r="B197" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C197" s="12" t="inlineStr">
         <is>
           <t>short</t>
         </is>
       </c>
-      <c r="D196" s="12" t="inlineStr">
+      <c r="D197" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock short</t>
         </is>
       </c>
-      <c r="E196" s="12" t="inlineStr">
+      <c r="E197" s="12" t="inlineStr">
         <is>
           <t>공매도 추이 조회</t>
         </is>
       </c>
-      <c r="F196" s="13" t="inlineStr">
+      <c r="F197" s="13" t="inlineStr">
         <is>
           <t>ka10014</t>
         </is>
       </c>
-      <c r="G196" s="12" t="inlineStr">
+      <c r="G197" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H196" s="12" t="inlineStr">
+      <c r="H197" s="12" t="inlineStr">
         <is>
           <t>--from (시작일자 (YYYYMMDD, 기본=30일전))
 --to (종료일자 (YYYYMMDD, 기본=오늘))</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B197" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C197" s="12" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="D197" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock sync</t>
-        </is>
-      </c>
-      <c r="E197" s="12" t="inlineStr">
-        <is>
-          <t>전 시장 종목 리스트를 다운받아 캐시에 저장</t>
-        </is>
-      </c>
-      <c r="F197" s="13" t="inlineStr">
-        <is>
-          <t>ka10099</t>
-        </is>
-      </c>
-      <c r="G197" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H197" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
     <row r="198">
       <c r="A198" s="12" t="inlineStr">
         <is>
@@ -8822,27 +8830,27 @@
       </c>
       <c r="C198" s="12" t="inlineStr">
         <is>
-          <t>tick-strength</t>
+          <t>sync</t>
         </is>
       </c>
       <c r="D198" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock tick-strength</t>
+          <t>kiwoom stock sync</t>
         </is>
       </c>
       <c r="E198" s="12" t="inlineStr">
         <is>
-          <t>체결강도추이 시간별</t>
+          <t>전 시장 종목 리스트를 다운받아 캐시에 저장</t>
         </is>
       </c>
       <c r="F198" s="13" t="inlineStr">
         <is>
-          <t>ka10046</t>
+          <t>ka10099</t>
         </is>
       </c>
       <c r="G198" s="12" t="inlineStr">
         <is>
-          <t>CODE (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H198" s="12" t="inlineStr">
@@ -8864,22 +8872,22 @@
       </c>
       <c r="C199" s="12" t="inlineStr">
         <is>
-          <t>timeprice</t>
+          <t>tick-strength</t>
         </is>
       </c>
       <c r="D199" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock timeprice</t>
+          <t>kiwoom stock tick-strength</t>
         </is>
       </c>
       <c r="E199" s="12" t="inlineStr">
         <is>
-          <t>시분 시세 조회</t>
+          <t>체결강도추이 시간별</t>
         </is>
       </c>
       <c r="F199" s="13" t="inlineStr">
         <is>
-          <t>ka10006</t>
+          <t>ka10046</t>
         </is>
       </c>
       <c r="G199" s="12" t="inlineStr">
@@ -8906,30 +8914,72 @@
       </c>
       <c r="C200" s="12" t="inlineStr">
         <is>
+          <t>timeprice</t>
+        </is>
+      </c>
+      <c r="D200" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock timeprice</t>
+        </is>
+      </c>
+      <c r="E200" s="12" t="inlineStr">
+        <is>
+          <t>시분 시세 조회</t>
+        </is>
+      </c>
+      <c r="F200" s="13" t="inlineStr">
+        <is>
+          <t>ka10006</t>
+        </is>
+      </c>
+      <c r="G200" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H200" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B201" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C201" s="12" t="inlineStr">
+        <is>
           <t>today-exec</t>
         </is>
       </c>
-      <c r="D200" s="12" t="inlineStr">
+      <c r="D201" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock today-exec</t>
         </is>
       </c>
-      <c r="E200" s="12" t="inlineStr">
+      <c r="E201" s="12" t="inlineStr">
         <is>
           <t>당일/전일 체결 조회</t>
         </is>
       </c>
-      <c r="F200" s="13" t="inlineStr">
+      <c r="F201" s="13" t="inlineStr">
         <is>
           <t>ka10084</t>
         </is>
       </c>
-      <c r="G200" s="12" t="inlineStr">
+      <c r="G201" s="12" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
         </is>
       </c>
-      <c r="H200" s="12" t="inlineStr">
+      <c r="H201" s="12" t="inlineStr">
         <is>
           <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))
 --mode [0, 1] (틱/분 (0=틱, 1=분))
@@ -8937,48 +8987,6 @@
         </is>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="12" t="inlineStr">
-        <is>
-          <t>stock</t>
-        </is>
-      </c>
-      <c r="B201" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C201" s="12" t="inlineStr">
-        <is>
-          <t>today-volume</t>
-        </is>
-      </c>
-      <c r="D201" s="12" t="inlineStr">
-        <is>
-          <t>kiwoom stock today-volume</t>
-        </is>
-      </c>
-      <c r="E201" s="12" t="inlineStr">
-        <is>
-          <t>당일/전일 체결량 조회</t>
-        </is>
-      </c>
-      <c r="F201" s="13" t="inlineStr">
-        <is>
-          <t>ka10055</t>
-        </is>
-      </c>
-      <c r="G201" s="12" t="inlineStr">
-        <is>
-          <t>CODE (필수)</t>
-        </is>
-      </c>
-      <c r="H201" s="12" t="inlineStr">
-        <is>
-          <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))</t>
-        </is>
-      </c>
-    </row>
     <row r="202">
       <c r="A202" s="12" t="inlineStr">
         <is>
@@ -8992,22 +9000,22 @@
       </c>
       <c r="C202" s="12" t="inlineStr">
         <is>
-          <t>trader</t>
+          <t>today-volume</t>
         </is>
       </c>
       <c r="D202" s="12" t="inlineStr">
         <is>
-          <t>kiwoom stock trader</t>
+          <t>kiwoom stock today-volume</t>
         </is>
       </c>
       <c r="E202" s="12" t="inlineStr">
         <is>
-          <t>거래원 조회</t>
+          <t>당일/전일 체결량 조회</t>
         </is>
       </c>
       <c r="F202" s="13" t="inlineStr">
         <is>
-          <t>ka10002</t>
+          <t>ka10055</t>
         </is>
       </c>
       <c r="G202" s="12" t="inlineStr">
@@ -9017,7 +9025,7 @@
       </c>
       <c r="H202" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--when [1, 2] 기본:1 (당일전일 (1=당일, 2=전일))</t>
         </is>
       </c>
     </row>
@@ -9034,70 +9042,74 @@
       </c>
       <c r="C203" s="12" t="inlineStr">
         <is>
+          <t>trader</t>
+        </is>
+      </c>
+      <c r="D203" s="12" t="inlineStr">
+        <is>
+          <t>kiwoom stock trader</t>
+        </is>
+      </c>
+      <c r="E203" s="12" t="inlineStr">
+        <is>
+          <t>거래원 조회</t>
+        </is>
+      </c>
+      <c r="F203" s="13" t="inlineStr">
+        <is>
+          <t>ka10002</t>
+        </is>
+      </c>
+      <c r="G203" s="12" t="inlineStr">
+        <is>
+          <t>CODE (필수)</t>
+        </is>
+      </c>
+      <c r="H203" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="12" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="B204" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C204" s="12" t="inlineStr">
+        <is>
           <t>watchlist</t>
         </is>
       </c>
-      <c r="D203" s="12" t="inlineStr">
+      <c r="D204" s="12" t="inlineStr">
         <is>
           <t>kiwoom stock watchlist</t>
         </is>
       </c>
-      <c r="E203" s="12" t="inlineStr">
+      <c r="E204" s="12" t="inlineStr">
         <is>
           <t>관심종목정보 조회 (코드를 |로 구분, 예: 005930|000660)</t>
         </is>
       </c>
-      <c r="F203" s="13" t="inlineStr">
+      <c r="F204" s="13" t="inlineStr">
         <is>
           <t>ka10095</t>
         </is>
       </c>
-      <c r="G203" s="12" t="inlineStr">
+      <c r="G204" s="12" t="inlineStr">
         <is>
           <t>CODES (필수)</t>
         </is>
       </c>
-      <c r="H203" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="14" t="inlineStr">
-        <is>
-          <t>stream</t>
-        </is>
-      </c>
-      <c r="B204" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C204" s="14" t="inlineStr">
-        <is>
-          <t>after-hours</t>
-        </is>
-      </c>
-      <c r="D204" s="14" t="inlineStr">
-        <is>
-          <t>kiwoom stream after-hours</t>
-        </is>
-      </c>
-      <c r="E204" s="14" t="inlineStr">
-        <is>
-          <t>주식시간외호가 실시간 (0E)</t>
-        </is>
-      </c>
-      <c r="F204" s="15" t="inlineStr"/>
-      <c r="G204" s="14" t="inlineStr">
-        <is>
-          <t>CODES (복수) (필수)</t>
-        </is>
-      </c>
-      <c r="H204" s="14" t="inlineStr">
-        <is>
-          <t>--raw (JSON 원본 출력)</t>
+      <c r="H204" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -9114,23 +9126,23 @@
       </c>
       <c r="C205" s="14" t="inlineStr">
         <is>
-          <t>balance</t>
+          <t>after-hours</t>
         </is>
       </c>
       <c r="D205" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream balance</t>
+          <t>kiwoom stream after-hours</t>
         </is>
       </c>
       <c r="E205" s="14" t="inlineStr">
         <is>
-          <t>잔고 실시간 (04)</t>
+          <t>주식시간외호가 실시간 (0E)</t>
         </is>
       </c>
       <c r="F205" s="15" t="inlineStr"/>
       <c r="G205" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H205" s="14" t="inlineStr">
@@ -9152,23 +9164,23 @@
       </c>
       <c r="C206" s="14" t="inlineStr">
         <is>
-          <t>best-bid</t>
+          <t>balance</t>
         </is>
       </c>
       <c r="D206" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream best-bid</t>
+          <t>kiwoom stream balance</t>
         </is>
       </c>
       <c r="E206" s="14" t="inlineStr">
         <is>
-          <t>주식우선호가 실시간 (0C)</t>
+          <t>잔고 실시간 (04)</t>
         </is>
       </c>
       <c r="F206" s="15" t="inlineStr"/>
       <c r="G206" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H206" s="14" t="inlineStr">
@@ -9190,64 +9202,64 @@
       </c>
       <c r="C207" s="14" t="inlineStr">
         <is>
-          <t>custom</t>
+          <t>best-bid</t>
         </is>
       </c>
       <c r="D207" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream custom</t>
+          <t>kiwoom stream best-bid</t>
         </is>
       </c>
       <c r="E207" s="14" t="inlineStr">
         <is>
-          <t>커스텀 실시간 타입으로 스트리밍</t>
+          <t>주식우선호가 실시간 (0C)</t>
         </is>
       </c>
       <c r="F207" s="15" t="inlineStr"/>
       <c r="G207" s="14" t="inlineStr">
         <is>
+          <t>CODES (복수) (필수)</t>
+        </is>
+      </c>
+      <c r="H207" s="14" t="inlineStr">
+        <is>
+          <t>--raw (JSON 원본 출력)</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="14" t="inlineStr">
+        <is>
+          <t>stream</t>
+        </is>
+      </c>
+      <c r="B208" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C208" s="14" t="inlineStr">
+        <is>
+          <t>custom</t>
+        </is>
+      </c>
+      <c r="D208" s="14" t="inlineStr">
+        <is>
+          <t>kiwoom stream custom</t>
+        </is>
+      </c>
+      <c r="E208" s="14" t="inlineStr">
+        <is>
+          <t>커스텀 실시간 타입으로 스트리밍</t>
+        </is>
+      </c>
+      <c r="F208" s="15" t="inlineStr"/>
+      <c r="G208" s="14" t="inlineStr">
+        <is>
           <t>TYPE_CODES (필수)
 CODES (복수) (선택)</t>
         </is>
       </c>
-      <c r="H207" s="14" t="inlineStr">
-        <is>
-          <t>--raw (JSON 원본 출력)</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="14" t="inlineStr">
-        <is>
-          <t>stream</t>
-        </is>
-      </c>
-      <c r="B208" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C208" s="14" t="inlineStr">
-        <is>
-          <t>elw-indicator</t>
-        </is>
-      </c>
-      <c r="D208" s="14" t="inlineStr">
-        <is>
-          <t>kiwoom stream elw-indicator</t>
-        </is>
-      </c>
-      <c r="E208" s="14" t="inlineStr">
-        <is>
-          <t>ELW 지표 실시간 (0u)</t>
-        </is>
-      </c>
-      <c r="F208" s="15" t="inlineStr"/>
-      <c r="G208" s="14" t="inlineStr">
-        <is>
-          <t>CODES (복수) (필수)</t>
-        </is>
-      </c>
       <c r="H208" s="14" t="inlineStr">
         <is>
           <t>--raw (JSON 원본 출력)</t>
@@ -9267,17 +9279,17 @@
       </c>
       <c r="C209" s="14" t="inlineStr">
         <is>
-          <t>elw-theory</t>
+          <t>elw-indicator</t>
         </is>
       </c>
       <c r="D209" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream elw-theory</t>
+          <t>kiwoom stream elw-indicator</t>
         </is>
       </c>
       <c r="E209" s="14" t="inlineStr">
         <is>
-          <t>ELW 이론가 실시간 (0m)</t>
+          <t>ELW 지표 실시간 (0u)</t>
         </is>
       </c>
       <c r="F209" s="15" t="inlineStr"/>
@@ -9305,17 +9317,17 @@
       </c>
       <c r="C210" s="14" t="inlineStr">
         <is>
-          <t>etf-nav</t>
+          <t>elw-theory</t>
         </is>
       </c>
       <c r="D210" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream etf-nav</t>
+          <t>kiwoom stream elw-theory</t>
         </is>
       </c>
       <c r="E210" s="14" t="inlineStr">
         <is>
-          <t>ETF NAV 실시간 (0G)</t>
+          <t>ELW 이론가 실시간 (0m)</t>
         </is>
       </c>
       <c r="F210" s="15" t="inlineStr"/>
@@ -9343,17 +9355,17 @@
       </c>
       <c r="C211" s="14" t="inlineStr">
         <is>
-          <t>expected</t>
+          <t>etf-nav</t>
         </is>
       </c>
       <c r="D211" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream expected</t>
+          <t>kiwoom stream etf-nav</t>
         </is>
       </c>
       <c r="E211" s="14" t="inlineStr">
         <is>
-          <t>주식예상체결 실시간 (0H)</t>
+          <t>ETF NAV 실시간 (0G)</t>
         </is>
       </c>
       <c r="F211" s="15" t="inlineStr"/>
@@ -9381,17 +9393,17 @@
       </c>
       <c r="C212" s="14" t="inlineStr">
         <is>
-          <t>gold</t>
+          <t>expected</t>
         </is>
       </c>
       <c r="D212" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream gold</t>
+          <t>kiwoom stream expected</t>
         </is>
       </c>
       <c r="E212" s="14" t="inlineStr">
         <is>
-          <t>국제금환산가격 실시간 (0I)</t>
+          <t>주식예상체결 실시간 (0H)</t>
         </is>
       </c>
       <c r="F212" s="15" t="inlineStr"/>
@@ -9419,23 +9431,23 @@
       </c>
       <c r="C213" s="14" t="inlineStr">
         <is>
-          <t>market-time</t>
+          <t>gold</t>
         </is>
       </c>
       <c r="D213" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream market-time</t>
+          <t>kiwoom stream gold</t>
         </is>
       </c>
       <c r="E213" s="14" t="inlineStr">
         <is>
-          <t>장시작시간 실시간 (0s)</t>
+          <t>국제금환산가격 실시간 (0I)</t>
         </is>
       </c>
       <c r="F213" s="15" t="inlineStr"/>
       <c r="G213" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H213" s="14" t="inlineStr">
@@ -9457,23 +9469,23 @@
       </c>
       <c r="C214" s="14" t="inlineStr">
         <is>
-          <t>multi</t>
+          <t>market-time</t>
         </is>
       </c>
       <c r="D214" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream multi</t>
+          <t>kiwoom stream market-time</t>
         </is>
       </c>
       <c r="E214" s="14" t="inlineStr">
         <is>
-          <t>주식체결+호가잔량 동시 스트리밍 (0B+0D)</t>
+          <t>장시작시간 실시간 (0s)</t>
         </is>
       </c>
       <c r="F214" s="15" t="inlineStr"/>
       <c r="G214" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H214" s="14" t="inlineStr">
@@ -9495,23 +9507,23 @@
       </c>
       <c r="C215" s="14" t="inlineStr">
         <is>
-          <t>order</t>
+          <t>multi</t>
         </is>
       </c>
       <c r="D215" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream order</t>
+          <t>kiwoom stream multi</t>
         </is>
       </c>
       <c r="E215" s="14" t="inlineStr">
         <is>
-          <t>주문체결 실시간 (00)</t>
+          <t>주식체결+호가잔량 동시 스트리밍 (0B+0D)</t>
         </is>
       </c>
       <c r="F215" s="15" t="inlineStr"/>
       <c r="G215" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H215" s="14" t="inlineStr">
@@ -9533,23 +9545,23 @@
       </c>
       <c r="C216" s="14" t="inlineStr">
         <is>
-          <t>orderbook</t>
+          <t>order</t>
         </is>
       </c>
       <c r="D216" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream orderbook</t>
+          <t>kiwoom stream order</t>
         </is>
       </c>
       <c r="E216" s="14" t="inlineStr">
         <is>
-          <t>주식호가잔량 실시간 (0D)</t>
+          <t>주문체결 실시간 (00)</t>
         </is>
       </c>
       <c r="F216" s="15" t="inlineStr"/>
       <c r="G216" s="14" t="inlineStr">
         <is>
-          <t>CODES (복수) (필수)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H216" s="14" t="inlineStr">
@@ -9571,17 +9583,17 @@
       </c>
       <c r="C217" s="14" t="inlineStr">
         <is>
-          <t>price</t>
+          <t>orderbook</t>
         </is>
       </c>
       <c r="D217" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream price</t>
+          <t>kiwoom stream orderbook</t>
         </is>
       </c>
       <c r="E217" s="14" t="inlineStr">
         <is>
-          <t>주식기세 실시간 (0A)</t>
+          <t>주식호가잔량 실시간 (0D)</t>
         </is>
       </c>
       <c r="F217" s="15" t="inlineStr"/>
@@ -9609,17 +9621,17 @@
       </c>
       <c r="C218" s="14" t="inlineStr">
         <is>
-          <t>program</t>
+          <t>price</t>
         </is>
       </c>
       <c r="D218" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream program</t>
+          <t>kiwoom stream price</t>
         </is>
       </c>
       <c r="E218" s="14" t="inlineStr">
         <is>
-          <t>종목프로그램매매 실시간 (0w)</t>
+          <t>주식기세 실시간 (0A)</t>
         </is>
       </c>
       <c r="F218" s="15" t="inlineStr"/>
@@ -9647,17 +9659,17 @@
       </c>
       <c r="C219" s="14" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>program</t>
         </is>
       </c>
       <c r="D219" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream quote</t>
+          <t>kiwoom stream program</t>
         </is>
       </c>
       <c r="E219" s="14" t="inlineStr">
         <is>
-          <t>주식체결 실시간 (0B)</t>
+          <t>종목프로그램매매 실시간 (0w)</t>
         </is>
       </c>
       <c r="F219" s="15" t="inlineStr"/>
@@ -9685,17 +9697,17 @@
       </c>
       <c r="C220" s="14" t="inlineStr">
         <is>
-          <t>sector-change</t>
+          <t>quote</t>
         </is>
       </c>
       <c r="D220" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream sector-change</t>
+          <t>kiwoom stream quote</t>
         </is>
       </c>
       <c r="E220" s="14" t="inlineStr">
         <is>
-          <t>업종등락 실시간 (0U)</t>
+          <t>주식체결 실시간 (0B)</t>
         </is>
       </c>
       <c r="F220" s="15" t="inlineStr"/>
@@ -9723,17 +9735,17 @@
       </c>
       <c r="C221" s="14" t="inlineStr">
         <is>
-          <t>sector-index</t>
+          <t>sector-change</t>
         </is>
       </c>
       <c r="D221" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream sector-index</t>
+          <t>kiwoom stream sector-change</t>
         </is>
       </c>
       <c r="E221" s="14" t="inlineStr">
         <is>
-          <t>업종지수 실시간 (0J)</t>
+          <t>업종등락 실시간 (0U)</t>
         </is>
       </c>
       <c r="F221" s="15" t="inlineStr"/>
@@ -9761,17 +9773,17 @@
       </c>
       <c r="C222" s="14" t="inlineStr">
         <is>
-          <t>stock-info</t>
+          <t>sector-index</t>
         </is>
       </c>
       <c r="D222" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream stock-info</t>
+          <t>kiwoom stream sector-index</t>
         </is>
       </c>
       <c r="E222" s="14" t="inlineStr">
         <is>
-          <t>주식종목정보 실시간 (0g)</t>
+          <t>업종지수 실시간 (0J)</t>
         </is>
       </c>
       <c r="F222" s="15" t="inlineStr"/>
@@ -9799,17 +9811,17 @@
       </c>
       <c r="C223" s="14" t="inlineStr">
         <is>
-          <t>trader</t>
+          <t>stock-info</t>
         </is>
       </c>
       <c r="D223" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream trader</t>
+          <t>kiwoom stream stock-info</t>
         </is>
       </c>
       <c r="E223" s="14" t="inlineStr">
         <is>
-          <t>주식당일거래원 실시간 (0F)</t>
+          <t>주식종목정보 실시간 (0g)</t>
         </is>
       </c>
       <c r="F223" s="15" t="inlineStr"/>
@@ -9837,28 +9849,28 @@
       </c>
       <c r="C224" s="14" t="inlineStr">
         <is>
-          <t>types</t>
+          <t>trader</t>
         </is>
       </c>
       <c r="D224" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream types</t>
+          <t>kiwoom stream trader</t>
         </is>
       </c>
       <c r="E224" s="14" t="inlineStr">
         <is>
-          <t>사용 가능한 실시간 타입 코드 목록</t>
+          <t>주식당일거래원 실시간 (0F)</t>
         </is>
       </c>
       <c r="F224" s="15" t="inlineStr"/>
       <c r="G224" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>CODES (복수) (필수)</t>
         </is>
       </c>
       <c r="H224" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--raw (JSON 원본 출력)</t>
         </is>
       </c>
     </row>
@@ -9875,71 +9887,109 @@
       </c>
       <c r="C225" s="14" t="inlineStr">
         <is>
-          <t>vi</t>
+          <t>types</t>
         </is>
       </c>
       <c r="D225" s="14" t="inlineStr">
         <is>
-          <t>kiwoom stream vi</t>
+          <t>kiwoom stream types</t>
         </is>
       </c>
       <c r="E225" s="14" t="inlineStr">
         <is>
-          <t>VI발동/해제 실시간 (1h)</t>
+          <t>사용 가능한 실시간 타입 코드 목록</t>
         </is>
       </c>
       <c r="F225" s="15" t="inlineStr"/>
       <c r="G225" s="14" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H225" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="14" t="inlineStr">
+        <is>
+          <t>stream</t>
+        </is>
+      </c>
+      <c r="B226" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C226" s="14" t="inlineStr">
+        <is>
+          <t>vi</t>
+        </is>
+      </c>
+      <c r="D226" s="14" t="inlineStr">
+        <is>
+          <t>kiwoom stream vi</t>
+        </is>
+      </c>
+      <c r="E226" s="14" t="inlineStr">
+        <is>
+          <t>VI발동/해제 실시간 (1h)</t>
+        </is>
+      </c>
+      <c r="F226" s="15" t="inlineStr"/>
+      <c r="G226" s="14" t="inlineStr">
+        <is>
           <t>CODES (복수) (필수)</t>
         </is>
       </c>
-      <c r="H225" s="14" t="inlineStr">
+      <c r="H226" s="14" t="inlineStr">
         <is>
           <t>--raw (JSON 원본 출력)</t>
         </is>
       </c>
     </row>
-    <row r="226">
-      <c r="A226" s="6" t="inlineStr">
+    <row r="227">
+      <c r="A227" s="6" t="inlineStr">
         <is>
           <t>watch</t>
         </is>
       </c>
-      <c r="B226" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C226" s="6" t="inlineStr">
+      <c r="B227" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C227" s="6" t="inlineStr">
         <is>
           <t>watch</t>
         </is>
       </c>
-      <c r="D226" s="6" t="inlineStr">
+      <c r="D227" s="6" t="inlineStr">
         <is>
           <t>kiwoom watch</t>
         </is>
       </c>
-      <c r="E226" s="6" t="inlineStr">
+      <c r="E227" s="6" t="inlineStr">
         <is>
           <t>실시간 종목 모니터링 (TUI 대시보드)</t>
         </is>
       </c>
-      <c r="F226" s="7" t="inlineStr"/>
-      <c r="G226" s="6" t="inlineStr">
+      <c r="F227" s="7" t="inlineStr"/>
+      <c r="G227" s="6" t="inlineStr">
         <is>
           <t>CODES (복수) (필수)</t>
         </is>
       </c>
-      <c r="H226" s="6" t="inlineStr">
+      <c r="H227" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H226"/>
+  <autoFilter ref="A1:H227"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10064,7 +10114,7 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
@@ -10139,7 +10189,7 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
release: bump version to 2.5.1
주문 안전 패치 (v2.5.0 전수 리뷰 Tier 1):
- 모든 주문 명령 미리보기 → 확인 순서 수정 (미국은 자동판별 거래소 표시 포함)
- --price 지정 + --type 미지정 = limit 추론, 시장가 계열 + 가격 = INVALID_INPUT
- 멱등성 fingerprint 바인딩 + IDEMPOTENCY_CONFLICT + 원장 파일 잠금
- account exchange apply confirm_gate 경유 (json CONFIRMATION_REQUIRED)
- 신용/금현물 --dry-run, --client-order-id 지원
- stream/watch --profile·KIWOOM_DOMAIN 존중, meta.env 단일 소스화

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$231</definedName>
@@ -5791,7 +5791,7 @@
       <c r="H128" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (시장가 주문시 생략, 미국주식은 소수점 4자리까지))
---type [after-hours, best, best-fok, best-ioc, conditional, first, fok, ioc, limit, loc, market, market-fok, market-ioc, mid, mid-fok, mid-ioc, moc, pre-market, single, stop, stop-limit, twap, twap-limit, vwap, vwap-limit] 기본:market (주문유형)
+--type [after-hours, best, best-fok, best-ioc, conditional, first, fok, ioc, limit, loc, market, market-fok, market-ioc, mid, mid-fok, mid-ioc, moc, pre-market, single, stop, stop-limit, twap, twap-limit, vwap, vwap-limit] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
 --exchange [KRX, NXT, SOR, nasdaq, nyse, amex] (거래소 (기본: 국내 KRX / 미국 자동판별))
 --cond-price (조건부가격 (국내 전용))
 --confirm (확인 프롬프트 없이 주문 실행)
@@ -6055,10 +6055,12 @@
       <c r="H134" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (시장가 주문시 생략))
---type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
+--type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (조건부가격)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6103,7 +6105,9 @@
         <is>
           <t>--qty (취소수량 (0=전량취소))
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6154,9 @@
         <is>
           <t>--exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (정정 조건부가격)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6194,10 +6200,12 @@
       <c r="H137" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (시장가 주문시 생략))
---type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
+--type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
 --exchange [KRX, NXT, SOR] 기본:KRX (거래소)
 --cond-price (조건부가격)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6283,8 +6291,10 @@
       <c r="H139" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (시장가 주문시 생략))
---type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6328,7 +6338,9 @@
       <c r="H140" s="12" t="inlineStr">
         <is>
           <t>--qty (취소수량 (0=전량취소))
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6541,7 +6553,9 @@
       </c>
       <c r="H145" s="12" t="inlineStr">
         <is>
-          <t>--confirm (확인 프롬프트 없이 주문 실행)</t>
+          <t>--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6627,8 +6641,10 @@
       <c r="H147" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (시장가 주문시 생략))
---type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
+--confirm (확인 프롬프트 없이 주문 실행)
+--dry-run (전송될 내용만 출력하고 주문을 전송하지 않음)
+--client-order-id (멱등성 키 (같은 키 재실행 시 재전송 없이 이전 응답 반환))</t>
         </is>
       </c>
     </row>
@@ -6714,7 +6730,7 @@
       <c r="H149" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (시장가 주문시 생략, 미국주식은 소수점 4자리까지))
---type [after-hours, best, best-fok, best-ioc, conditional, first, fok, ioc, limit, loc, market, market-fok, market-ioc, mid, mid-fok, mid-ioc, moc, pre-market, single, stop, stop-limit, twap, twap-limit, vwap, vwap-limit] 기본:market (주문유형)
+--type [after-hours, best, best-fok, best-ioc, conditional, first, fok, ioc, limit, loc, market, market-fok, market-ioc, mid, mid-fok, mid-ioc, moc, pre-market, single, stop, stop-limit, twap, twap-limit, vwap, vwap-limit] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
 --exchange [KRX, NXT, SOR, nasdaq, nyse, amex] (거래소 (기본: 국내 KRX / 미국 자동판별))
 --cond-price (조건부가격 (국내 전용))
 --stop (STOP가격 (미국 stop/stop-limit 전용))

</xml_diff>

<commit_message>
release: bump version to 2.6.0
에이전트 계약 강화 (Tier-2):
- 전역 --next-key/--all-pages 페이지네이션
- fail_input 입력오류 envelope 전면화 (~30개 지점)
- TOKEN_EXPIRED(8005) exit 2 → 3, httpx 타임아웃 → NETWORK_ERROR
- describe --paths/--depth, market 명령 API ID 노출
- config setup 비대화형 지원, stream 엣지 경로 계약 준수
- meta.fields_unmatched, LEDGER_BUSY, validate --price/--type 규칙
- README 예제 오류 수정 (-f json 위치), Excel 재생성

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -2162,9 +2162,9 @@
           <t>--profile 기본:default (프로필 이름)
 --appkey (키움 API App Key)
 --secretkey (키움 API Secret Key)
---domain [prod, mock] 기본:mock (도메인)
+--domain [prod, mock] (도메인)
 --account (계좌번호)
---token-storage [keychain, env] 기본:keychain (접근토큰 저장 방식)</t>
+--token-storage [keychain, env] (접근토큰 저장 방식)</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,8 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>--paths (경로+한줄설명 평면 목록만 출력 (전체 트리 대비 토큰 절약 — 발견용))
+--depth (하위 명령 재귀 깊이 제한 (예: --depth 1 = 한 단계만))</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2470,11 @@
           <t>ELW 잔량 순위</t>
         </is>
       </c>
-      <c r="F46" s="11" t="inlineStr"/>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>ka30010</t>
+        </is>
+      </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2509,7 +2514,11 @@
           <t>거래원별 ELW 순매매 상위</t>
         </is>
       </c>
-      <c r="F47" s="11" t="inlineStr"/>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>ka30002</t>
+        </is>
+      </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2551,7 +2560,11 @@
           <t>ELW 등락율 순위</t>
         </is>
       </c>
-      <c r="F48" s="11" t="inlineStr"/>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>ka30009</t>
+        </is>
+      </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2591,7 +2604,11 @@
           <t>ELW 종목 상세정보</t>
         </is>
       </c>
-      <c r="F49" s="11" t="inlineStr"/>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>ka30012</t>
+        </is>
+      </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -2629,7 +2646,11 @@
           <t>ELW 괴리율</t>
         </is>
       </c>
-      <c r="F50" s="11" t="inlineStr"/>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>ka30004</t>
+        </is>
+      </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2671,7 +2692,11 @@
           <t>ELW LP 보유 일별 추이</t>
         </is>
       </c>
-      <c r="F51" s="11" t="inlineStr"/>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>ka30003</t>
+        </is>
+      </c>
       <c r="G51" s="10" t="inlineStr">
         <is>
           <t>UNDERLYING_CODE (필수)</t>
@@ -2709,7 +2734,11 @@
           <t>ELW 근접율</t>
         </is>
       </c>
-      <c r="F52" s="11" t="inlineStr"/>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>ka30011</t>
+        </is>
+      </c>
       <c r="G52" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -2747,7 +2776,11 @@
           <t>ELW 조건 검색</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr"/>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>ka30005</t>
+        </is>
+      </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2789,7 +2822,11 @@
           <t>ELW 민감도 지표</t>
         </is>
       </c>
-      <c r="F54" s="11" t="inlineStr"/>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>ka10050</t>
+        </is>
+      </c>
       <c r="G54" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -2827,7 +2864,11 @@
           <t>ELW 일별 민감도 지표</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr"/>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>ka10048</t>
+        </is>
+      </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -2865,7 +2906,11 @@
           <t>ELW 가격 급등락</t>
         </is>
       </c>
-      <c r="F56" s="11" t="inlineStr"/>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>ka30001</t>
+        </is>
+      </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2911,7 +2956,11 @@
           <t>ETF 전체 시세</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr"/>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>ka40004</t>
+        </is>
+      </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -2954,7 +3003,11 @@
           <t>ETF 일별추이</t>
         </is>
       </c>
-      <c r="F58" s="11" t="inlineStr"/>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>ka40003</t>
+        </is>
+      </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -2992,7 +3045,11 @@
           <t>ETF 일자별 체결</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr"/>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>ka40008</t>
+        </is>
+      </c>
       <c r="G59" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3030,7 +3087,11 @@
           <t>ETF 종목정보</t>
         </is>
       </c>
-      <c r="F60" s="11" t="inlineStr"/>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>ka40002</t>
+        </is>
+      </c>
       <c r="G60" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3068,7 +3129,11 @@
           <t>ETF 수익율 조회</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr"/>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>ka40001</t>
+        </is>
+      </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3107,7 +3172,11 @@
           <t>ETF 시간대별 체결</t>
         </is>
       </c>
-      <c r="F62" s="11" t="inlineStr"/>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>ka40007</t>
+        </is>
+      </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3145,7 +3214,11 @@
           <t>ETF 시간대별 체결 (상세)</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr"/>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>ka40009</t>
+        </is>
+      </c>
       <c r="G63" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3183,7 +3256,11 @@
           <t>ETF 시간대별 추이</t>
         </is>
       </c>
-      <c r="F64" s="11" t="inlineStr"/>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>ka40006</t>
+        </is>
+      </c>
       <c r="G64" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3221,7 +3298,11 @@
           <t>ETF 시간대별 추이 (상세)</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr"/>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>ka40010</t>
+        </is>
+      </c>
       <c r="G65" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3259,7 +3340,11 @@
           <t>금현물 일봉 차트</t>
         </is>
       </c>
-      <c r="F66" s="11" t="inlineStr"/>
+      <c r="F66" s="11" t="inlineStr">
+        <is>
+          <t>ka50081</t>
+        </is>
+      </c>
       <c r="G66" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3299,7 +3384,11 @@
           <t>금현물 분봉 차트</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr"/>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>ka50080</t>
+        </is>
+      </c>
       <c r="G67" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3339,7 +3428,11 @@
           <t>금현물 월봉 차트</t>
         </is>
       </c>
-      <c r="F68" s="11" t="inlineStr"/>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>ka50083</t>
+        </is>
+      </c>
       <c r="G68" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3379,7 +3472,11 @@
           <t>금현물 틱차트</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr"/>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>ka50079</t>
+        </is>
+      </c>
       <c r="G69" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3419,7 +3516,11 @@
           <t>금현물 주봉 차트</t>
         </is>
       </c>
-      <c r="F70" s="11" t="inlineStr"/>
+      <c r="F70" s="11" t="inlineStr">
+        <is>
+          <t>ka50082</t>
+        </is>
+      </c>
       <c r="G70" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3459,7 +3560,11 @@
           <t>금현물 일별 추이</t>
         </is>
       </c>
-      <c r="F71" s="11" t="inlineStr"/>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>ka50012</t>
+        </is>
+      </c>
       <c r="G71" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3498,7 +3603,11 @@
           <t>금현물 체결 추이</t>
         </is>
       </c>
-      <c r="F72" s="11" t="inlineStr"/>
+      <c r="F72" s="11" t="inlineStr">
+        <is>
+          <t>ka50010</t>
+        </is>
+      </c>
       <c r="G72" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3536,7 +3645,11 @@
           <t>금현물 예상 체결</t>
         </is>
       </c>
-      <c r="F73" s="11" t="inlineStr"/>
+      <c r="F73" s="11" t="inlineStr">
+        <is>
+          <t>ka50087</t>
+        </is>
+      </c>
       <c r="G73" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3574,7 +3687,11 @@
           <t>금현물 투자자 현황</t>
         </is>
       </c>
-      <c r="F74" s="11" t="inlineStr"/>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>ka52301</t>
+        </is>
+      </c>
       <c r="G74" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3612,7 +3729,11 @@
           <t>금현물 호가</t>
         </is>
       </c>
-      <c r="F75" s="11" t="inlineStr"/>
+      <c r="F75" s="11" t="inlineStr">
+        <is>
+          <t>ka50101</t>
+        </is>
+      </c>
       <c r="G75" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3651,7 +3772,11 @@
           <t>금현물 시세정보</t>
         </is>
       </c>
-      <c r="F76" s="11" t="inlineStr"/>
+      <c r="F76" s="11" t="inlineStr">
+        <is>
+          <t>ka50100</t>
+        </is>
+      </c>
       <c r="G76" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3689,7 +3814,11 @@
           <t>금현물 당일 분봉 차트</t>
         </is>
       </c>
-      <c r="F77" s="11" t="inlineStr"/>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>ka50092</t>
+        </is>
+      </c>
       <c r="G77" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3728,7 +3857,11 @@
           <t>금현물 당일 틱차트</t>
         </is>
       </c>
-      <c r="F78" s="11" t="inlineStr"/>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>ka50091</t>
+        </is>
+      </c>
       <c r="G78" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3767,7 +3900,11 @@
           <t>프로그램매매 차익잔고 추이</t>
         </is>
       </c>
-      <c r="F79" s="11" t="inlineStr"/>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t>ka90006</t>
+        </is>
+      </c>
       <c r="G79" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3806,7 +3943,11 @@
           <t>프로그램매매 누적 추이</t>
         </is>
       </c>
-      <c r="F80" s="11" t="inlineStr"/>
+      <c r="F80" s="11" t="inlineStr">
+        <is>
+          <t>ka90007</t>
+        </is>
+      </c>
       <c r="G80" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3847,7 +3988,11 @@
           <t>프로그램매매 추이 (일자별)</t>
         </is>
       </c>
-      <c r="F81" s="11" t="inlineStr"/>
+      <c r="F81" s="11" t="inlineStr">
+        <is>
+          <t>ka90010</t>
+        </is>
+      </c>
       <c r="G81" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -3889,7 +4034,11 @@
           <t>종목 일별 프로그램매매 추이</t>
         </is>
       </c>
-      <c r="F82" s="11" t="inlineStr"/>
+      <c r="F82" s="11" t="inlineStr">
+        <is>
+          <t>ka90013</t>
+        </is>
+      </c>
       <c r="G82" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3928,7 +4077,11 @@
           <t>종목 시간별 프로그램매매 추이</t>
         </is>
       </c>
-      <c r="F83" s="11" t="inlineStr"/>
+      <c r="F83" s="11" t="inlineStr">
+        <is>
+          <t>ka90008</t>
+        </is>
+      </c>
       <c r="G83" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -3967,7 +4120,11 @@
           <t>프로그램매매 추이 (시간대별)</t>
         </is>
       </c>
-      <c r="F84" s="11" t="inlineStr"/>
+      <c r="F84" s="11" t="inlineStr">
+        <is>
+          <t>ka90005</t>
+        </is>
+      </c>
       <c r="G84" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4009,7 +4166,11 @@
           <t>시간외 단일가 등락율 순위</t>
         </is>
       </c>
-      <c r="F85" s="11" t="inlineStr"/>
+      <c r="F85" s="11" t="inlineStr">
+        <is>
+          <t>ka10098</t>
+        </is>
+      </c>
       <c r="G85" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4052,7 +4213,11 @@
           <t>거래대금 상위</t>
         </is>
       </c>
-      <c r="F86" s="11" t="inlineStr"/>
+      <c r="F86" s="11" t="inlineStr">
+        <is>
+          <t>ka10032</t>
+        </is>
+      </c>
       <c r="G86" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4092,7 +4257,11 @@
           <t>잔량율 급증</t>
         </is>
       </c>
-      <c r="F87" s="11" t="inlineStr"/>
+      <c r="F87" s="11" t="inlineStr">
+        <is>
+          <t>ka10022</t>
+        </is>
+      </c>
       <c r="G87" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4135,7 +4304,11 @@
           <t>종목별 증권사 순위</t>
         </is>
       </c>
-      <c r="F88" s="11" t="inlineStr"/>
+      <c r="F88" s="11" t="inlineStr">
+        <is>
+          <t>ka10038</t>
+        </is>
+      </c>
       <c r="G88" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -4176,7 +4349,11 @@
           <t>증권사별 매매 상위</t>
         </is>
       </c>
-      <c r="F89" s="11" t="inlineStr"/>
+      <c r="F89" s="11" t="inlineStr">
+        <is>
+          <t>ka10039</t>
+        </is>
+      </c>
       <c r="G89" s="10" t="inlineStr">
         <is>
           <t>BROKER_CODE (필수)</t>
@@ -4217,7 +4394,11 @@
           <t>전일대비 등락률 상위</t>
         </is>
       </c>
-      <c r="F90" s="11" t="inlineStr"/>
+      <c r="F90" s="11" t="inlineStr">
+        <is>
+          <t>ka10027</t>
+        </is>
+      </c>
       <c r="G90" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4263,7 +4444,11 @@
           <t>신용비율 상위</t>
         </is>
       </c>
-      <c r="F91" s="11" t="inlineStr"/>
+      <c r="F91" s="11" t="inlineStr">
+        <is>
+          <t>ka10033</t>
+        </is>
+      </c>
       <c r="G91" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4306,7 +4491,11 @@
           <t>예상체결 등락률 상위</t>
         </is>
       </c>
-      <c r="F92" s="11" t="inlineStr"/>
+      <c r="F92" s="11" t="inlineStr">
+        <is>
+          <t>ka10029</t>
+        </is>
+      </c>
       <c r="G92" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4350,7 +4539,11 @@
           <t>외국계 창구 매매 상위</t>
         </is>
       </c>
-      <c r="F93" s="11" t="inlineStr"/>
+      <c r="F93" s="11" t="inlineStr">
+        <is>
+          <t>ka10037</t>
+        </is>
+      </c>
       <c r="G93" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4392,7 +4585,11 @@
           <t>외인 연속 순매매 상위</t>
         </is>
       </c>
-      <c r="F94" s="11" t="inlineStr"/>
+      <c r="F94" s="11" t="inlineStr">
+        <is>
+          <t>ka10035</t>
+        </is>
+      </c>
       <c r="G94" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4433,7 +4630,11 @@
           <t>외인 한도소진율 증가 상위</t>
         </is>
       </c>
-      <c r="F95" s="11" t="inlineStr"/>
+      <c r="F95" s="11" t="inlineStr">
+        <is>
+          <t>ka10036</t>
+        </is>
+      </c>
       <c r="G95" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4473,7 +4674,11 @@
           <t>외국인/기관 매매 상위</t>
         </is>
       </c>
-      <c r="F96" s="11" t="inlineStr"/>
+      <c r="F96" s="11" t="inlineStr">
+        <is>
+          <t>ka90009</t>
+        </is>
+      </c>
       <c r="G96" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4515,7 +4720,11 @@
           <t>외인 기간별 매매 상위</t>
         </is>
       </c>
-      <c r="F97" s="11" t="inlineStr"/>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>ka10034</t>
+        </is>
+      </c>
       <c r="G97" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4556,7 +4765,11 @@
           <t>실시간 종목 조회 순위</t>
         </is>
       </c>
-      <c r="F98" s="11" t="inlineStr"/>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>ka00198</t>
+        </is>
+      </c>
       <c r="G98" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4594,7 +4807,11 @@
           <t>장중 투자자별 매매 상위</t>
         </is>
       </c>
-      <c r="F99" s="11" t="inlineStr"/>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>ka10065</t>
+        </is>
+      </c>
       <c r="G99" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4635,7 +4852,11 @@
           <t>상하한가 순위</t>
         </is>
       </c>
-      <c r="F100" s="11" t="inlineStr"/>
+      <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>ka10017</t>
+        </is>
+      </c>
       <c r="G100" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4680,7 +4901,11 @@
           <t>당일 주요 거래원</t>
         </is>
       </c>
-      <c r="F101" s="11" t="inlineStr"/>
+      <c r="F101" s="11" t="inlineStr">
+        <is>
+          <t>ka10040</t>
+        </is>
+      </c>
       <c r="G101" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -4718,7 +4943,11 @@
           <t>고저가근접 순위</t>
         </is>
       </c>
-      <c r="F102" s="11" t="inlineStr"/>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>ka10018</t>
+        </is>
+      </c>
       <c r="G102" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4762,7 +4991,11 @@
           <t>순매수 거래원 순위</t>
         </is>
       </c>
-      <c r="F103" s="11" t="inlineStr"/>
+      <c r="F103" s="11" t="inlineStr">
+        <is>
+          <t>ka10042</t>
+        </is>
+      </c>
       <c r="G103" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -4805,7 +5038,11 @@
           <t>신고저가 순위</t>
         </is>
       </c>
-      <c r="F104" s="11" t="inlineStr"/>
+      <c r="F104" s="11" t="inlineStr">
+        <is>
+          <t>ka10016</t>
+        </is>
+      </c>
       <c r="G104" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4851,7 +5088,11 @@
           <t>호가잔량 급증</t>
         </is>
       </c>
-      <c r="F105" s="11" t="inlineStr"/>
+      <c r="F105" s="11" t="inlineStr">
+        <is>
+          <t>ka10021</t>
+        </is>
+      </c>
       <c r="G105" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4895,7 +5136,11 @@
           <t>호가잔량 상위</t>
         </is>
       </c>
-      <c r="F106" s="11" t="inlineStr"/>
+      <c r="F106" s="11" t="inlineStr">
+        <is>
+          <t>ka10020</t>
+        </is>
+      </c>
       <c r="G106" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4938,7 +5183,11 @@
           <t>전일 거래량 상위</t>
         </is>
       </c>
-      <c r="F107" s="11" t="inlineStr"/>
+      <c r="F107" s="11" t="inlineStr">
+        <is>
+          <t>ka10031</t>
+        </is>
+      </c>
       <c r="G107" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -4980,7 +5229,11 @@
           <t>동일 순매매 순위</t>
         </is>
       </c>
-      <c r="F108" s="11" t="inlineStr"/>
+      <c r="F108" s="11" t="inlineStr">
+        <is>
+          <t>ka10062</t>
+        </is>
+      </c>
       <c r="G108" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5024,7 +5277,11 @@
           <t>가격급등락 순위</t>
         </is>
       </c>
-      <c r="F109" s="11" t="inlineStr"/>
+      <c r="F109" s="11" t="inlineStr">
+        <is>
+          <t>ka10019</t>
+        </is>
+      </c>
       <c r="G109" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5071,7 +5328,11 @@
           <t>당일 상위 이탈원</t>
         </is>
       </c>
-      <c r="F110" s="11" t="inlineStr"/>
+      <c r="F110" s="11" t="inlineStr">
+        <is>
+          <t>ka10053</t>
+        </is>
+      </c>
       <c r="G110" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -5109,7 +5370,11 @@
           <t>당일 거래량 상위</t>
         </is>
       </c>
-      <c r="F111" s="11" t="inlineStr"/>
+      <c r="F111" s="11" t="inlineStr">
+        <is>
+          <t>ka10030</t>
+        </is>
+      </c>
       <c r="G111" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5155,7 +5420,11 @@
           <t>거래량 급증</t>
         </is>
       </c>
-      <c r="F112" s="11" t="inlineStr"/>
+      <c r="F112" s="11" t="inlineStr">
+        <is>
+          <t>ka10023</t>
+        </is>
+      </c>
       <c r="G112" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5200,7 +5469,11 @@
           <t>업종 일봉 차트</t>
         </is>
       </c>
-      <c r="F113" s="11" t="inlineStr"/>
+      <c r="F113" s="11" t="inlineStr">
+        <is>
+          <t>ka20006</t>
+        </is>
+      </c>
       <c r="G113" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5238,7 +5511,11 @@
           <t>업종 분봉 차트</t>
         </is>
       </c>
-      <c r="F114" s="11" t="inlineStr"/>
+      <c r="F114" s="11" t="inlineStr">
+        <is>
+          <t>ka20005</t>
+        </is>
+      </c>
       <c r="G114" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5277,7 +5554,11 @@
           <t>업종 월봉 차트</t>
         </is>
       </c>
-      <c r="F115" s="11" t="inlineStr"/>
+      <c r="F115" s="11" t="inlineStr">
+        <is>
+          <t>ka20008</t>
+        </is>
+      </c>
       <c r="G115" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5315,7 +5596,11 @@
           <t>업종 틱차트</t>
         </is>
       </c>
-      <c r="F116" s="11" t="inlineStr"/>
+      <c r="F116" s="11" t="inlineStr">
+        <is>
+          <t>ka20004</t>
+        </is>
+      </c>
       <c r="G116" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5353,7 +5638,11 @@
           <t>업종 주봉 차트</t>
         </is>
       </c>
-      <c r="F117" s="11" t="inlineStr"/>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>ka20007</t>
+        </is>
+      </c>
       <c r="G117" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5391,7 +5680,11 @@
           <t>업종 년봉 차트</t>
         </is>
       </c>
-      <c r="F118" s="11" t="inlineStr"/>
+      <c r="F118" s="11" t="inlineStr">
+        <is>
+          <t>ka20019</t>
+        </is>
+      </c>
       <c r="G118" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5429,7 +5722,11 @@
           <t>업종코드 리스트</t>
         </is>
       </c>
-      <c r="F119" s="11" t="inlineStr"/>
+      <c r="F119" s="11" t="inlineStr">
+        <is>
+          <t>ka10101</t>
+        </is>
+      </c>
       <c r="G119" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5467,7 +5764,11 @@
           <t>업종 현재가 조회</t>
         </is>
       </c>
-      <c r="F120" s="11" t="inlineStr"/>
+      <c r="F120" s="11" t="inlineStr">
+        <is>
+          <t>ka20001</t>
+        </is>
+      </c>
       <c r="G120" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5505,7 +5806,11 @@
           <t>업종 현재가 일별</t>
         </is>
       </c>
-      <c r="F121" s="11" t="inlineStr"/>
+      <c r="F121" s="11" t="inlineStr">
+        <is>
+          <t>ka20009</t>
+        </is>
+      </c>
       <c r="G121" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5543,7 +5848,11 @@
           <t>전업종 지수</t>
         </is>
       </c>
-      <c r="F122" s="11" t="inlineStr"/>
+      <c r="F122" s="11" t="inlineStr">
+        <is>
+          <t>ka20003</t>
+        </is>
+      </c>
       <c r="G122" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5581,7 +5890,11 @@
           <t>업종별 투자자 순매수</t>
         </is>
       </c>
-      <c r="F123" s="11" t="inlineStr"/>
+      <c r="F123" s="11" t="inlineStr">
+        <is>
+          <t>ka10051</t>
+        </is>
+      </c>
       <c r="G123" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5622,7 +5935,11 @@
           <t>업종 프로그램매매</t>
         </is>
       </c>
-      <c r="F124" s="11" t="inlineStr"/>
+      <c r="F124" s="11" t="inlineStr">
+        <is>
+          <t>ka10010</t>
+        </is>
+      </c>
       <c r="G124" s="10" t="inlineStr">
         <is>
           <t>CODE (필수)</t>
@@ -5660,7 +5977,11 @@
           <t>업종별 주가</t>
         </is>
       </c>
-      <c r="F125" s="11" t="inlineStr"/>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>ka20002</t>
+        </is>
+      </c>
       <c r="G125" s="10" t="inlineStr">
         <is>
           <t>INDS_CD (필수)</t>
@@ -5699,7 +6020,11 @@
           <t>테마 그룹별 조회</t>
         </is>
       </c>
-      <c r="F126" s="11" t="inlineStr"/>
+      <c r="F126" s="11" t="inlineStr">
+        <is>
+          <t>ka90001</t>
+        </is>
+      </c>
       <c r="G126" s="10" t="inlineStr">
         <is>
           <t>-</t>
@@ -5742,7 +6067,11 @@
           <t>테마 구성종목 조회</t>
         </is>
       </c>
-      <c r="F127" s="11" t="inlineStr"/>
+      <c r="F127" s="11" t="inlineStr">
+        <is>
+          <t>ka90002</t>
+        </is>
+      </c>
       <c r="G127" s="10" t="inlineStr">
         <is>
           <t>THEME_CODE (필수)</t>
@@ -6777,7 +7106,7 @@
       <c r="H150" s="12" t="inlineStr">
         <is>
           <t>--price (주문가격 (생략 시 현재가로 예상비용 계산))
---type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] 기본:market (주문유형)
+--type [limit, market, conditional, after-hours, pre-market, single, best, first, ioc, market-ioc, best-ioc, fok, market-fok, best-fok, stop, mid, mid-ioc, mid-fok] (주문유형 (기본: --price 지정 시 limit, 미지정 시 market))
 --exchange [KRX, NXT] 기본:KRX (거래소)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
release: bump version to 2.9.0
트랜치 A (실제 돈·틀린 숫자) 23커밋. 531 -> 699 tests.

patch가 아닌 minor인 이유: _ABS_FIELDS/_SIGNED_FIELDS 편입분이 normalize.py를
거쳐 -f json 타입을 바꾼다 (26개 필드 문자열 -> 숫자 + <필드>_direction 키).
저장소 선례상 json 형태 변경은 v2.3.0·v2.5.0 모두 minor였고, patch 릴리스가
json 계약을 바꾼 적은 없다.

Excel 재생성분은 이번 브랜치와 무관한 v2.7.0/v2.8.0 드리프트 4행 (help 텍스트
전용). v2.9.0의 --price 가드는 click.Choice가 아닌 교차검증이라 이 워크북
포맷에는 구조적으로 드러나지 않는다.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kiwoom_cli_commands.xlsx
+++ b/kiwoom_cli_commands.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="요약" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체 명령어" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'전체 명령어'!$A$1:$H$232</definedName>
@@ -1930,7 +1930,8 @@
       <c r="H32" s="4" t="inlineStr">
         <is>
           <t>--raw (JSON 원본 출력)
---next-key (연속조회 커서 (이전 응답의 meta.cont.next_key))</t>
+--next-key (연속조회 커서 (이전 응답의 meta.cont.next_key))
+--confirm (주문성 API(매수/매도/정정/취소/환전) 확인 생략 (자동화용))</t>
         </is>
       </c>
     </row>
@@ -6291,7 +6292,7 @@
       <c r="H132" s="12" t="inlineStr">
         <is>
           <t>--exchange [K] 기본:K (거래소 (K=KRX))
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 조건검색 실시간 등록 실행)</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6337,7 @@
           <t>--exchange [K] 기본:K (거래소 (K=KRX))
 --cont-yn (연속조회여부)
 --next-key (연속조회키)
---confirm (확인 프롬프트 없이 주문 실행)</t>
+--confirm (확인 프롬프트 없이 조건검색 조회 실행)</t>
         </is>
       </c>
     </row>
@@ -6378,7 +6379,7 @@
       </c>
       <c r="H134" s="12" t="inlineStr">
         <is>
-          <t>--confirm (확인 프롬프트 없이 주문 실행)</t>
+          <t>--confirm (확인 프롬프트 없이 조건검색 실시간 해제 실행)</t>
         </is>
       </c>
     </row>

</xml_diff>